<commit_message>
docs: document solutions and update status
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -534,7 +534,7 @@
         <is>
           <t>1. local database (sqlite) initialized on first launch
 2. schema migration with version tracking
-3. defined folder layout inside app data dir (db, library, logs, cache)</t>
+3. defined layout inside app data dir (database.sqlite, library, logs, cache)</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
   - documented for reuse
 2. implement the application shell with homepage
 3. i18n and theming infrastructure ready for all screens
-4. future features shown as disabled / "coming soon" in navigation</t>
+4. future features stay navigable and open a "Coming soon" page</t>
         </is>
       </c>
     </row>
@@ -649,16 +649,16 @@
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>Settings screen for general configuration. Language (VN/EN) and theme (light/dark/system) changes apply immediately. When the app data directory changes, the app checks write permission first, then asks the user whether to move existing data or start with an empty folder. The Pipeline section sets the maximum number of concurrent pipelines. Settings are saved in a JSON file at %ProgramData%/DreamerStudio.</t>
+          <t>Settings screen for general configuration. Language (VN/EN) and theme (light/dark) changes apply immediately. When the app data directory changes, the app checks write permission first, then asks the user whether to move existing data or start with an empty folder. The Pipeline section sets the maximum number of concurrent pipelines. Settings are saved in a JSON file at %LOCALAPPDATA%/DreamerStudio.</t>
         </is>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
           <t>1. setting screen with General, Storage, and Pipeline sections
-2. able to change language (VN/EN) and theme (light/dark/system)
+2. able to change language (VN/EN) and theme (light/dark)
 3. able to change app data directory, with write-permission check and data migration option
 4. able to set max concurrent pipelines
-5. settings saved in %ProgramData%/DreamerStudio/settings.json</t>
+5. settings saved in %LOCALAPPDATA%/DreamerStudio/settings.json</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>AC-1. SQLite database file is created in &lt;app data&gt;/db on first launch
+          <t>AC-1. SQLite database file is created at &lt;app data&gt;/database.sqlite on first launch
 AC-2. Features access data only through the shared data access layer
 AC-3. Database connection errors are logged and can be checked by Diagnostics</t>
         </is>
@@ -1753,7 +1753,7 @@
         <is>
           <t>AC-1. Current schema version is stored in the database
 AC-2. Pending migrations run automatically on startup, in order
-AC-3. A failed migration is rolled back, logged, and reported to the user</t>
+AC-3. A failed migration is logged, shown to the user in an error dialog, and the app quits</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>Define and create the standard folders inside the app data directory (db, library, logs, cache). All features get paths from a single path resolver, so changing the app data directory (TH02-01) works everywhere.</t>
+          <t>Define and create the standard folders inside the app data directory (library, logs, cache); the database file sits at the app data root (TSK-005). All features get paths from a single path resolver, so changing the app data directory (TH02-01) works everywhere.</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
@@ -1795,8 +1795,8 @@
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Default app data directory is %ProgramData%/DreamerStudio
-AC-2. Folders db, library, logs, cache are created on first launch
+          <t>AC-1. Default app data directory is %LOCALAPPDATA%/DreamerStudio
+AC-2. Folders library, logs, cache are created on first launch
 AC-3. Missing folders are recreated automatically on startup
 AC-4. All features resolve paths through a single path resolver</t>
         </is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Set up the i18n framework with VN/EN translation files for all screens. Navigation items of features not yet released are shown as placeholders.</t>
+          <t>Set up the i18n framework with VN/EN translation files for all screens. Navigation items of features not yet released stay navigable and open a "Coming soon" page.</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
@@ -1899,7 +1899,7 @@
           <t>AC-1. All UI text comes from translation files (VN, EN), no hard-coded strings
 AC-2. Language can be switched at runtime without restarting the app
 AC-3. Missing translation keys fall back to English
-AC-4. Navigation items of unreleased features are disabled with a "Coming soon" label</t>
+AC-4. Navigation items of unreleased features stay enabled; opening one shows a "Coming soon" page in the content area (feature name, short description, planned release)</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,9 @@
 AC-2. Header and content area follow the main layout from the design system
 AC-3. App shell provides a running-pipelines indicator slot and a toast notification area
 AC-4. Homepage shows quick shortcuts and a recent pipelines section (empty state when no data)
-AC-5. App applies the light/dark/system theme at runtime</t>
+AC-5. App applies the light/dark theme at runtime
+AC-6. Homepage shows status cards for the app data folder (path, open in Explorer), the AI backend state and the running pipelines (empty until the pipeline executor exists)
+AC-7. Status bar shows the app data folder, the running-pipelines indicator and the AI backend state while it is starting or failed</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2420,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Settings screen opened from the sidebar, grouped into General, Storage, and Pipeline sections. Settings are validated before saving to %ProgramData%/DreamerStudio/settings.json.</t>
+          <t>Settings screen opened from the sidebar, grouped into General, Storage, and Pipeline sections. Settings are validated before saving to %LOCALAPPDATA%/DreamerStudio/settings.json.</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -2434,7 +2436,7 @@
       <c r="H2" s="1" t="inlineStr">
         <is>
           <t>AC-1. Settings screen is opened from the sidebar and has General, Storage, and Pipeline sections
-AC-2. Settings are saved to %ProgramData%/DreamerStudio/settings.json and persist across restarts
+AC-2. Settings are saved to %LOCALAPPDATA%/DreamerStudio/settings.json and persist across restarts
 AC-3. Invalid values are rejected with a clear message
 AC-4. Each section can be reset to default values</t>
         </is>
@@ -2463,7 +2465,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>In the General section, the user switches the UI language (VN/EN) and theme (light/dark/system). Changes apply immediately without restarting.</t>
+          <t>In the General section, the user switches the UI language (VN/EN) and theme (light/dark). Changes apply immediately without restarting.</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -2479,9 +2481,8 @@
       <c r="H3" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can switch language between VN and EN; the UI updates immediately
-AC-2. User can switch theme between light, dark, and system; the UI updates immediately
-AC-3. System theme follows Windows theme changes while the app is running
-AC-4. On first launch, language follows the OS language and falls back to English</t>
+AC-2. User can switch theme between light and dark; the UI updates immediately
+AC-3. On first launch, settings.json is created with the defaults: light theme and English</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2509,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>In the Storage section, the user sees the current app data directory and can move it to another folder, with checks and a choice to move existing data or start empty.</t>
+          <t>In the Storage section, the user sees the current app data directory and can move it to another folder, with checks and a choice to move existing data or start empty. Moving covers database.sqlite, library, logs and cache; settings.json stays in place (TSK-010).</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -2554,7 +2555,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Application settings (language, theme, app data directory path, pipeline settings) are stored in %ProgramData%/DreamerStudio/settings.json. The file stays at this fixed location, outside the configurable app data directory, so the app can always find it at startup.</t>
+          <t>Application settings (language, theme, app data directory path, pipeline settings) are stored in %LOCALAPPDATA%/DreamerStudio/settings.json. The file stays at this fixed location, outside the configurable app data directory, so the app can always find it at startup.</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -2569,8 +2570,8 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Settings are read from %ProgramData%/DreamerStudio/settings.json at startup
-AC-2. Missing file is created with default values; default app data directory is %ProgramData%/DreamerStudio
+          <t>AC-1. Settings are read from %LOCALAPPDATA%/DreamerStudio/settings.json at startup
+AC-2. Missing file is created with default values; default app data directory is %LOCALAPPDATA%/DreamerStudio
 AC-3. Invalid or corrupted file falls back to default values, is logged, and the user is notified
 AC-4. If the configured app data directory is missing or unreachable, the app warns and lets the user pick another folder or use the default</t>
         </is>
@@ -2715,7 +2716,7 @@
         <is>
           <t>AC-1. Each check returns OK/Warning/Error, a message, and a suggested fix
 AC-2. New checks can be registered without changing the engine
-AC-3. Built-in check: read &amp; write permission on the app data directory (default %ProgramData%/DreamerStudio)
+AC-3. Built-in check: read &amp; write permission on the app data directory (default %LOCALAPPDATA%/DreamerStudio)
 AC-4. TODO: more checks will be defined once the architecture is ready (TSK-001)</t>
         </is>
       </c>
@@ -4111,7 +4112,7 @@
       <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Local database for pipeline history, library metadata, bookmarks.
-Risk [unverified]: node:sqlite is experimental in Node; require('node:sqlite') was broken in some Electron releases (fixed in 36.7.3 / 37.2.3 / 38). Pin Electron and prove it in a TSK-002 spike.</t>
+Risk (resolved 2026-10-17): node:sqlite is experimental in Node; require('node:sqlite') was broken in some Electron releases (fixed in 36.7.3 / 37.2.3 / 38). Electron is pinned to 44.9.0 and the TSK-002 spike proves it.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -4141,7 +4142,7 @@
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>Initial ADR from the human.</t>
+          <t>Initial ADR from the human. Verified 2026-10-17: electron/main/app/sqlite-spike.ts opens an in-memory DatabaseSync in Electron 44.9.0 main and logs SQLite 3.53.4.</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
@@ -4682,7 +4683,7 @@
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>Human chose the recommended option. Follow-up: update TH02-01, TSK-007, TSK-010, REQ-006, TSK-011 via /solo-analysis.</t>
+          <t>Human chose the recommended option. Follow-up: update TH02-01, TSK-007, TSK-010, REQ-006, TSK-011 via /solo-analysis. Follow-up done on 2026-10-17.</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr">
@@ -4863,7 +4864,7 @@
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>Human decision. Follow-up: update TSK-005 AC-1 (database path) and TSK-007 AC-2 (folders library, logs, cache) via /solo-analysis.</t>
+          <t>Human decision. Follow-up: update TSK-005 AC-1 (database path) and TSK-007 AC-2 (folders library, logs, cache) via /solo-analysis. Follow-up done on 2026-10-17.</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(TSK002): Initialize project codebase following structure and tech stack
- fix(app): resolve human reviews for development setup
- fix(app): resolve review and test findings [TSK-002]
- docs(repo): document dev, lint, format and test commands [TSK-002]
- feat(app): add electron, angular and backend skeleton with app version [TSK-002]
- chore(repo): add workspace, lint, format and test tooling [TSK-002]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -3926,7 +3926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4873,21 +4873,75 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n"/>
-      <c r="B20" s="1" t="n"/>
-      <c r="C20" s="1" t="n"/>
-      <c r="D20" s="1" t="n"/>
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="n"/>
-      <c r="G20" s="1" t="n"/>
-      <c r="H20" s="1" t="n"/>
-      <c r="I20" s="1" t="n"/>
-      <c r="J20" s="1" t="n"/>
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>AD-19</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Build and dev tool for main + preload</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>Electron main and preload are TypeScript and need a bundle; dev mode must run Angular, rebuild main and restart Electron (TH01-01 solution Q-01).</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>TH01-01, TSK-002, TSK-004</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>esbuild + scripts/dev.mjs — Fast, small config · one dev script for ng serve, esbuild watch and Electron
+tsc only — No bundler · Cons: no bundling of shared/, manual restart
+electron-vite — All-in-one · Cons: Vite for the renderer conflicts with Angular CLI</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>esbuild + scripts/dev.mjs</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>esbuild + scripts/dev.mjs</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-01 on 2026-10-17. Built in TSK-002: electron/esbuild.mjs (CJS bundles, APP_VERSION define), scripts/dev.mjs.</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="n"/>
+      <c r="D21" s="1" t="n"/>
+      <c r="E21" s="1" t="n"/>
+      <c r="F21" s="1" t="n"/>
+      <c r="G21" s="1" t="n"/>
+      <c r="H21" s="1" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(TSK003): Centralize logging and catch unhandled errors
- docs(logging): document logging and error handling [TSK-003]
- fix(logging): resolve review and test findings [TSK-003]
- feat(backend): add backend logging, errors and lifecycle [TSK-003]
- feat(logging): add main logger and UI error handling [TSK-003]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -1602,7 +1602,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
-          <t>Human chose the recommended option.</t>
+          <t>Human chose the recommended option. Built in TSK-003 with Q-04 (daily, keep 7 days): main-YYYY-MM-DD.log (main + renderer) and backend-YYYY-MM-DD.log; same line format ISO UTC · level · process · module · message; each process deletes its own files older than 7 days.</t>
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr">
@@ -4928,21 +4928,75 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n"/>
-      <c r="B21" s="1" t="n"/>
-      <c r="C21" s="1" t="n"/>
-      <c r="D21" s="1" t="n"/>
-      <c r="E21" s="1" t="n"/>
-      <c r="F21" s="1" t="n"/>
-      <c r="G21" s="1" t="n"/>
-      <c r="H21" s="1" t="n"/>
-      <c r="I21" s="1" t="n"/>
-      <c r="J21" s="1" t="n"/>
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>AD-20</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Logger in Electron main</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>Main needs a file logger with a custom line format and dated files; the renderer logs through main (TH01-01 solution Q-02).</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>TH01-01, TSK-003</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>electron-log — Main only, renderer via typed log:write IPC · custom format and resolvePathFn
+In-house logger — No dependency · Cons: write own file handling
+pino — Fast, structured · Cons: JSON lines, extra transports for files</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>electron-log</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>electron-log</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-02 on 2026-10-17. Built in TSK-003: electron/main/logging (electron-log 5.4.4). resolvePathFn is called on every write, so files switch at midnight; maxSize 0.</t>
+        </is>
+      </c>
+      <c r="J21" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
+      <c r="E22" s="1" t="n"/>
+      <c r="F22" s="1" t="n"/>
+      <c r="G22" s="1" t="n"/>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(TSK004): Build the app into a portable Windows package
- docs(build): document portable Windows build [TSK-004]
- fix(build): resolve review and test findings [TSK-004]
- feat(build): add portable Windows package [TSK-004]

 Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -1647,7 +1647,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4522,7 +4522,7 @@
       </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
-          <t>Human chose the recommended option.</t>
+          <t>Human chose the recommended option. Built in TSK-004: backend/backend.spec (one-folder dreamer-backend, no UPX, console exe started hidden so stderr reaches the main log); node scripts/py.mjs freeze. VCRUNTIME140 DLLs are bundled.</t>
         </is>
       </c>
       <c r="J11" s="1" t="inlineStr">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
-          <t>Human chose the recommended option.</t>
+          <t>Human chose the recommended option. Built in TSK-004: electron/electron-builder.config.mjs (zip, x64, extraResources renderer + backend), scripts/build.mjs, pnpm package → dist/DreamerStudio-&lt;version&gt;-win-x64.zip. No node_modules in the package: main and preload are bundled by esbuild.</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
@@ -4982,21 +4982,74 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n"/>
-      <c r="B22" s="1" t="n"/>
-      <c r="C22" s="1" t="n"/>
-      <c r="D22" s="1" t="n"/>
-      <c r="E22" s="1" t="n"/>
-      <c r="F22" s="1" t="n"/>
-      <c r="G22" s="1" t="n"/>
-      <c r="H22" s="1" t="n"/>
-      <c r="I22" s="1" t="n"/>
-      <c r="J22" s="1" t="n"/>
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>AD-21</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Target Windows architecture</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>The portable package must run on Windows 10/11 (TSK-004 AC-2); every target arch needs its own Electron and frozen Python build (TH01-01 solution Q-05).</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>TH01-01, TSK-004</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>x64 only — One build, matches the dev machine and most PCs
+x64 + arm64 — Native on ARM laptops · Cons: two builds, arm64 Python wheels and a test machine needed</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>x64 only</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>x64 only</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-05 on 2026-10-17. Target Windows 10 22H2 / 11 x64. Built in TSK-004: win target zip, arch x64, file name ends with -win-x64.zip.</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="1" t="n"/>
+      <c r="C23" s="1" t="n"/>
+      <c r="D23" s="1" t="n"/>
+      <c r="E23" s="1" t="n"/>
+      <c r="F23" s="1" t="n"/>
+      <c r="G23" s="1" t="n"/>
+      <c r="H23" s="1" t="n"/>
+      <c r="I23" s="1" t="n"/>
+      <c r="J23" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(TSK005): Set up SQLite as the local database
- docs(storage): document database and data access layer [TSK-005]
- fix(storage): resolve review and test findings [TSK-005]
- feat(storage): add SQLite database and data access layer [TSK-005]
- refactor(storage): resolve app data paths once and add fatal data dialog [TSK-005]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>Initial ADR from the human. Verified 2026-10-17: electron/main/app/sqlite-spike.ts opens an in-memory DatabaseSync in Electron 44.9.0 main and logs SQLite 3.53.4.</t>
+          <t>Initial ADR from the human. Verified 2026-10-17 with the TSK-002 spike: DatabaseSync in Electron 44.9.0 main, SQLite 3.53.4. Built in TSK-005 (2026-10-18): electron/main/storage/database.ts opens &lt;app data&gt;/database.sqlite, no ExperimentalWarning; the spike was removed.</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
@@ -5035,21 +5035,74 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n"/>
-      <c r="B23" s="1" t="n"/>
-      <c r="C23" s="1" t="n"/>
-      <c r="D23" s="1" t="n"/>
-      <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="n"/>
-      <c r="G23" s="1" t="n"/>
-      <c r="H23" s="1" t="n"/>
-      <c r="I23" s="1" t="n"/>
-      <c r="J23" s="1" t="n"/>
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>AD-22</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Data access style</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>TSK-005 needs one shared data access layer over node:sqlite in main (AD-03, AD-04). TH01-02 solution Q-03.</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>TH01-02, TSK-005, TSK-006, TSK-008, TSK-013</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Raw SQL + thin typed wrapper — Database class (get/all/run/exec/transaction) and one repository per table; no dependency · Cons: SQL strings unchecked by the compiler
+Query builder (Kysely) — Typed queries · Cons: extra dependency and a node:sqlite dialect to maintain</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Raw SQL + thin typed wrapper</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>Raw SQL + thin typed wrapper</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-03 on 2026-10-17. Built in TSK-005: electron/main/storage/database.ts; features import repositories only, enforced by ESLint no-restricted-imports.</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="1" t="n"/>
+      <c r="C24" s="1" t="n"/>
+      <c r="D24" s="1" t="n"/>
+      <c r="E24" s="1" t="n"/>
+      <c r="F24" s="1" t="n"/>
+      <c r="G24" s="1" t="n"/>
+      <c r="H24" s="1" t="n"/>
+      <c r="I24" s="1" t="n"/>
+      <c r="J24" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(TSK006): Upgrade the database schema safely between releases
- docs(storage): document schema migrations [TSK-006]
- fix(storage): resolve review and test findings [TSK-006]
- feat(storage): run schema migrations on startup [TSK-006]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -1746,7 +1746,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5088,21 +5088,180 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
-      <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="n"/>
-      <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="1" t="n"/>
-      <c r="J24" s="1" t="n"/>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>AD-23</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Schema version storage</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>TSK-006 AC-1 needs the current schema version in the database. TH01-02 solution Q-01.</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>TH01-02, TSK-006</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Migration history table — one row per applied file (id, version, upgrade_num, applied_at); shows what ran and when
+PRAGMA user_version — built in, one integer · Cons: no history, no file names</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>Migration history table</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>Migration history table</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-01 on 2026-10-17; table named sys_migration_history and created by the first migration 0.0.0_0__sys_migration_history_table.sql (human, 2026-10-18). Built in TSK-006: electron/main/storage/migrator.ts.</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>AD-24</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>Migration file format</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>TSK-006 AC-2 runs pending migrations in order on startup. TH01-02 solution Q-02.</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>TH01-02, TSK-006, TH01-04, TSK-013</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>.sql files — &lt;version&gt;_&lt;upgrade_num&gt;__&lt;name&gt;.sql; plain SQL, shipped as extraResources
+TS modules — can run code · Cons: bundled into main, harder to review as SQL</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>.sql files</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>.sql files</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-02 on 2026-10-17; __&lt;name&gt; suffix and upgrade_num from 0 added 2026-10-18. Sorted by major, minor, patch, upgrade_num as numbers. A released file is never edited; a fix ships as a new file. Packaged at &lt;resources&gt;/migrations.</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>AD-25</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>Backup before migrating</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>A failed migration is not rolled back (TSK-006 AC-3), so the data may be left half-upgraded. TH01-02 solution Q-04.</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>TH01-02, TSK-006</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>One backup — VACUUM INTO database.backup.sqlite before pending migrations, when rows exist; overwritten each time
+No backup — simplest · Cons: a failed migration leaves no way back</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>One backup</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>One backup</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-04 on 2026-10-17. Built in TSK-006: the DB_MIGRATION_FAILED dialog names the backup when one exists.</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+      <c r="E27" s="1" t="n"/>
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="n"/>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(TSK007): Define the folder layout inside the app data directory
- docs(storage): document app data folders and single instance [TSK-007]
- fix(storage): resolve review and test findings [TSK-007]
- feat(storage): create app data folders and allow one instance [TSK-007]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(REQ001): Utilize the storybook to define design system, app shell, and homepage
- feat(design): match the main layout to the app shell and add resizable panels [REQ-001]
- docs(design): document the design system and Storybook [REQ-001]
- fix(design): resolve review and test findings [REQ-001]
- feat(design): add layout pattern stories [REQ-001]
- feat(design): add base components with stories [REQ-001]
- feat(design): add tokens, icons and Storybook [REQ-001]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -1845,7 +1845,7 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5247,21 +5247,180 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n"/>
-      <c r="B27" s="1" t="n"/>
-      <c r="C27" s="1" t="n"/>
-      <c r="D27" s="1" t="n"/>
-      <c r="E27" s="1" t="n"/>
-      <c r="F27" s="1" t="n"/>
-      <c r="G27" s="1" t="n"/>
-      <c r="H27" s="1" t="n"/>
-      <c r="I27" s="1" t="n"/>
-      <c r="J27" s="1" t="n"/>
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>AD-26</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>How much Bootstrap</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>TH01-03 needs one design system from DESIGN.md tokens. TH01-03 solution Q-02.</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>TH01-03, REQ-001, REQ-003</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Reboot + utilities — spacers mapped to --sp-*, --bs-* mapped to tokens; own components from tokens
+Bootstrap components themed — less code · Cons: fights the tokens, heavier CSS</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>Reboot + utilities</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>Reboot + utilities</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-02 on 2026-10-17. Built in REQ-001: angular/src/styles/_bootstrap.scss (reboot, root, helpers, utilities; color/opacity utilities removed); Sass import deprecations silenced in angular.json.</t>
+        </is>
+      </c>
+      <c r="J27" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>AD-27</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>Fonts</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>Inter and Source Serif 4 must ship with the app (CSP font-src 'self') and cover Vietnamese. TH01-03 solution Q-05.</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>TH01-03, REQ-001</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>npm @fontsource-variable — pinned packages, woff2 bundled by the Angular build
+woff2 files by hand — no dependency · Cons: manual updates</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>npm @fontsource-variable</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>npm @fontsource-variable</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-05 on 2026-10-17. Built in REQ-001: @fontsource-variable/inter 5.3.0, @fontsource-variable/source-serif-4 5.3.1; _fonts.scss declares families Inter and Source Serif 4 (latin, latin-ext, vietnamese).</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>AD-28</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>Storybook location and imports</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>REQ-001 AC-1 needs Storybook for Angular 22 with stories for tokens, components and layouts.</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>TH01-03, REQ-001, REQ-003</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>angular/stories + @components alias — stories apart from the code, imports via @components/*
+Stories next to components — default layout · Cons: mixes docs and code</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>angular/stories + @components alias</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>angular/stories + @components alias</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>Human decided on 2026-10-18 (REQ-001). @storybook/angular 10.6.2 (webpack builder, needs @angular-devkit/build-angular); stories *.stories.ts under foundations/, components/, layout/; pnpm storybook.</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n"/>
+      <c r="B30" s="1" t="n"/>
+      <c r="C30" s="1" t="n"/>
+      <c r="D30" s="1" t="n"/>
+      <c r="E30" s="1" t="n"/>
+      <c r="F30" s="1" t="n"/>
+      <c r="G30" s="1" t="n"/>
+      <c r="H30" s="1" t="n"/>
+      <c r="I30" s="1" t="n"/>
+      <c r="J30" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REQ002): Set up i18n and show upcoming features as placeholders
- docs(i18n): document translation files and language switch [REQ-002]
- feat(i18n): translate the shell, homepage and Coming soon [REQ-002]
- feat(i18n): add translation files, lookup and language IPC [REQ-002]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -3927,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5406,21 +5406,74 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n"/>
-      <c r="B30" s="1" t="n"/>
-      <c r="C30" s="1" t="n"/>
-      <c r="D30" s="1" t="n"/>
-      <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="n"/>
-      <c r="G30" s="1" t="n"/>
-      <c r="H30" s="1" t="n"/>
-      <c r="I30" s="1" t="n"/>
-      <c r="J30" s="1" t="n"/>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>AD-29</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Where the translation files live</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>REQ-002 needs one set of VN/EN texts for the renderer and the native dialogs in main (D-10). TH01-03 solution Q-04.</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>TH01-03, REQ-002</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>shared/i18n — one pair of files imported at build time by Angular and esbuild; one translate() lookup
+angular/src/assets/i18n — served to the renderer · Cons: main reads files at runtime, second loader</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>shared/i18n</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>shared/i18n</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-04 on 2026-10-17. Built in REQ-002: shared/i18n/{en,vi}.json (flat dotted keys) + translate.ts; resolveJsonModule; I18nService/t pipe (renderer), MainI18n (main), app:set-language; scripts/check-i18n.mjs in pnpm lint.</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="1" t="n"/>
+      <c r="C31" s="1" t="n"/>
+      <c r="D31" s="1" t="n"/>
+      <c r="E31" s="1" t="n"/>
+      <c r="F31" s="1" t="n"/>
+      <c r="G31" s="1" t="n"/>
+      <c r="H31" s="1" t="n"/>
+      <c r="I31" s="1" t="n"/>
+      <c r="J31" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(solu): define solution for module TH01-04
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Executor to start, stop, monitor the background pipelines</t>
+          <t>Executor to start, cancel, monitor the background pipelines</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>1. start, stop, monitor a background pipeline
+          <t>1. start, cancel, monitor a background pipeline
 2. pipeline history management (view, delete)
 3. a demo pipeline to validate the executor
 4. running pipelines marked as cancelled after app restart
@@ -1979,7 +1979,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>Run, stop, and track background pipelines</t>
+          <t>Run, cancel, and track background pipelines</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -2000,11 +2000,13 @@
       <c r="H15" s="1" t="inlineStr">
         <is>
           <t>AC-1. Pipelines run in the background without blocking the UI
-AC-2. Status transitions: queued -&gt; running -&gt; succeeded / failed / cancelled
+AC-2. Status transitions: queued -&gt; running -&gt; succeeded / failed / cancelled; queued -&gt; cancelled
 AC-3. Each run reports progress, current step, and writes its own log
-AC-4. A running pipeline can be stopped safely
+AC-4. A queued or running pipeline can be cancelled safely: a running one stops at the next checkpoint and its cleanup runs
 AC-5. Concurrent pipelines are limited at 1
-AC-6. Runs are stored in the database; runs left running are marked as cancelled after restart</t>
+AC-6. Runs are stored in the database; runs left queued or running after a restart are marked as cancelled
+AC-7. On app quit, queued and running runs are cancelled and stored as cancelled before the app exits
+AC-8. A run's log file is kept until the run is deleted</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2072,7 @@
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>Let users start, stop, and monitor running pipelines</t>
+          <t>Let users start, cancel, and monitor running pipelines</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -2090,9 +2092,9 @@
       </c>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Running-pipelines indicator in the app shell shows the number of running pipelines
-AC-2. Pipeline screen lists running pipelines with status, progress, and current step
-AC-3. User can start and stop a pipeline from the UI
+          <t>AC-1. Running-pipelines indicator in the app shell shows the number of active runs (running + queued); it is hidden or shows zero when none are active
+AC-2. Pipeline screen lists active runs (running and queued) with status, progress, and current step
+AC-3. User can start and cancel a pipeline from the UI
 AC-4. User can open a pipeline to view its live log
 AC-5. Toast notification when a pipeline succeeds or fails, click to open its details</t>
         </is>
@@ -2139,7 +2141,7 @@
           <t>AC-1. History lists finished runs with type, status, start/end time, and duration
 AC-2. User can filter runs by status and pipeline type
 AC-3. User can view the details and log of a past run
-AC-4. User can delete one or many runs after confirmation; related log files are deleted too
+AC-4. User can delete one or many finished runs after confirmation; related log files are deleted too
 AC-5. Homepage recent pipelines section shows the latest runs</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat(TSK008): Run, cancel, and track background pipelines
- docs(pipelines): document the pipeline executor [TSK-008]
- fix(pipelines): resolve review and test findings [TSK-008]
- feat(pipelines): run pipelines in the background [TSK-008]
- feat(pipelines): add pipeline run storage and IPC contract [TSK-008]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -1994,7 +1994,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -3929,7 +3929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5461,21 +5461,180 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
-      <c r="H31" s="1" t="n"/>
-      <c r="I31" s="1" t="n"/>
-      <c r="J31" s="1" t="n"/>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>AD-30</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>How the live run log reaches the renderer</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>REQ-004 AC-4 shows a run's log live. TH01-04 solution Q-01.</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>TH01-04, TSK-008, REQ-004, REQ-005</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Push events (pipeline:log) — main batches new lines every 250 ms per run; renderer loads the file once with pipeline:get-log
+Poll the file — Cons: delay, repeated reads</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>Push events (pipeline:log)</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>Push events (pipeline:log)</t>
+        </is>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-01 on 2026-10-19. Built in TSK-008: RunLog (electron/main/pipelines/run-log.ts) broadcasts PipelineLogChunk { runId, lines }.</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>AD-31</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline run ID</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Run IDs appear in the URL /pipelines/&lt;id&gt;, the log file name and the UI. TH01-04 solution Q-02.</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>TH01-04, TSK-008, REQ-004, REQ-005</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>UUID text — crypto.randomUUID(); display "{type} #{first 8 chars}"
+INTEGER AUTOINCREMENT — Cons: guessable, reused after a reset</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>UUID text</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>UUID text</t>
+        </is>
+      </c>
+      <c r="H32" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-02 on 2026-10-19. Built in TSK-008: pipeline_run.id TEXT PRIMARY KEY; log &lt;app data&gt;/logs/pipelines/&lt;id&gt;.log.</t>
+        </is>
+      </c>
+      <c r="J32" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>AD-32</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>How much pipeline history is loaded</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>REQ-005 AC-1 lists finished runs; history grows without automatic cleanup. TH01-04 solution Q-03.</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>TH01-04, TSK-008, REQ-005</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Pages of 50 + Load more — keyset cursor (created_at, id), total with the same filters
+Newest 200, no paging — Cons: older runs unreachable</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>Pages of 50 + Load more</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>Pages of 50 + Load more</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-03 on 2026-10-19. Built in TSK-008: PipelineRunRepository.list (keyset, filters bound as JSON via json_each), pipeline:list.</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="n"/>
+      <c r="D34" s="1" t="n"/>
+      <c r="E34" s="1" t="n"/>
+      <c r="F34" s="1" t="n"/>
+      <c r="G34" s="1" t="n"/>
+      <c r="H34" s="1" t="n"/>
+      <c r="I34" s="1" t="n"/>
+      <c r="J34" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(TSK009,REQ004): Demo pipeline and pipeline monitor
- docs(pipelines): document the demo pipeline and pipeline monitor [REQ-004]
- fix(pipelines): resolve review and test findings [REQ-004]
- feat(pipelines): add the pipelines page with details and live log [REQ-004]
- feat(pipelines): track pipelines in the shell [REQ-004]
- feat(components): add tabs, progress kinds and a dense table [REQ-004]
- feat(pipelines): add the demo pipeline and backend jobs [TSK-009]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
@@ -3929,7 +3929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5620,21 +5620,180 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n"/>
-      <c r="B34" s="1" t="n"/>
-      <c r="C34" s="1" t="n"/>
-      <c r="D34" s="1" t="n"/>
-      <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="n"/>
-      <c r="G34" s="1" t="n"/>
-      <c r="H34" s="1" t="n"/>
-      <c r="I34" s="1" t="n"/>
-      <c r="J34" s="1" t="n"/>
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>AD-33</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>Does the demo pipeline call the Python backend</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>TSK-009 demo validates the executor; AD-05 says Python runs heavy steps. TH01-04 solution Q-04.</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>TH01-04, TSK-009</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>Step 3 as a backend job — proves main → Python progress, log and cancel end to end
+Node-only demo — Cons: backend path unproven until 0.1.0</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>Step 3 as a backend job</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>Step 3 as a backend job</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-04 on 2026-10-19. Built in TSK-009: demo-pipeline.ts step 3 calls runBackendJob('demo'); backend/app/jobs/demo.py.</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>AD-34</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>How main runs a backend job (progress, log, cancel)</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline steps in Python must report progress and log lines and stop on Cancel. TH01-04 solution Q-07.</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>TH01-04, TSK-009, AD-05</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>One streaming request (NDJSON) — cancel = abort the fetch; Python stops on disconnect; no job state
+Job resource + SSE — Cons: job state in Python (against AD-04), more endpoints</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>One streaming request (NDJSON)</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>One streaming request (NDJSON)</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-07 on 2026-10-19. Built in TSK-009: POST /jobs/{type} (application/x-ndjson: progress, log, done, error); electron/main/backend/backend-job.ts runBackendJob; disconnect verified through the token middleware.</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>AD-35</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>IPC error convention for invoke calls</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>Electron passes only the message of an error thrown in ipcMain.handle, so CodedError.code was lost in the renderer (TSK-008 finding 4); the pipelines UI needs PIPELINE_NOT_FOUND and BACKEND_UNAVAILABLE.</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>TSK-008, TSK-009, REQ-004, all IPC</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Result envelope — handlers return { value } | { error: AppError }; the preload rejects with the AppError
+JSON in the error message — Cons: fragile string parsing in the preload</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>Result envelope</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Result envelope</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>Human chose the recommendation on 2026-10-19 (D-1). Built in TSK-009: electron/main/ipc/handle.ts, shared/ipc/ipc-result.ts, preload call(), isAppError, AppErrorHandler uses the code.</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="n"/>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="1" t="n"/>
+      <c r="J37" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REQ005): Let users view and clean up past pipeline runs
- docs(pipelines): document the pipeline history [REQ-005]
- fix(pipelines): resolve review and test findings [REQ-005]
- refactor(stories): render the real pipelines page in stories [REQ-005]
- feat(pipelines): add the pipeline history [REQ-005]
- feat(pipelines): keep recent runs live and delete runs [REQ-005]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">

</xml_diff>

<commit_message>
chore(solu): define solution for module settings
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -649,14 +649,14 @@
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>Settings screen for general configuration. Language (VN/EN) and theme (light/dark) changes apply immediately. When the app data directory changes, the app checks write permission first, then asks the user whether to move existing data or start with an empty folder. The Pipeline section sets the maximum number of concurrent pipelines. Settings are saved in a JSON file at %LOCALAPPDATA%/DreamerStudio.</t>
+          <t>Settings screen for general configuration. Language (VN/EN) and theme (light/dark) changes apply immediately. The user can open another folder as the app data directory: existing data there is opened, otherwise new data is created; the switch applies without restarting. The Pipeline section sets the maximum number of concurrent pipelines. Settings are saved in a JSON file at %LOCALAPPDATA%/DreamerStudio.</t>
         </is>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>1. setting screen with General, Storage, and Pipeline sections
+          <t>1. setting screen with General, Storage, and Pipeline sections; Diagnostics and About (TH02-02) are in the same screen
 2. able to change language (VN/EN) and theme (light/dark)
-3. able to change app data directory, with write-permission check and data migration option
+3. able to open another app data directory (existing or new data), applied without restart
 4. able to set max concurrent pipelines
 5. settings saved in %LOCALAPPDATA%/DreamerStudio/settings.json</t>
         </is>
@@ -691,14 +691,13 @@
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>The About page shows the app name, version, build date, license, and repository link. The Diagnostics page runs self-checks; each check returns OK/Warning/Error with a suggested fix. Release 0.0.0 checks read &amp; write permission on the app data directory; more checks will be defined once the architecture is ready.</t>
+          <t>The About page shows the app name, version, build date, license, and repository link. The Diagnostics page runs self-checks; each check returns OK/Warning/Error with a suggested fix. Diagnostics are stateless: results are returned directly and nothing is saved. Release 0.0.0 checks app data read &amp; write, database integrity, AI backend, settings file and free disk space.</t>
         </is>
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
           <t>1. show current application version and about information
-2. self-check read &amp; write permission on app data directory (more checks TBD after architecture)
-3. export diagnostics report with logs</t>
+2. self-check app data permission, database, AI backend, settings file, disk space; results shown directly, nothing saved</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2002,7 @@
 AC-2. Status transitions: queued -&gt; running -&gt; succeeded / failed / cancelled; queued -&gt; cancelled
 AC-3. Each run reports progress, current step, and writes its own log
 AC-4. A queued or running pipeline can be cancelled safely: a running one stops at the next checkpoint and its cleanup runs
-AC-5. Concurrent pipelines are limited at 1
+AC-5. Concurrent pipelines are limited by the max concurrency setting (REQ-009, default 1)
 AC-6. Runs are stored in the database; runs left queued or running after a restart are marked as cancelled
 AC-7. On app quit, queued and running runs are cancelled and stored as cancelled before the app exits
 AC-8. A run's log file is kept until the run is deleted</t>
@@ -2437,10 +2436,10 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Settings screen is opened from the sidebar and has General, Storage, and Pipeline sections
-AC-2. Settings are saved to %LOCALAPPDATA%/DreamerStudio/settings.json and persist across restarts
+          <t>AC-1. Settings screen is opened from the sidebar and has General, Storage, and Pipeline sections; Diagnostics and About (TH02-02) are in the same screen
+AC-2. Each valid change is saved at once (no Save button) to %LOCALAPPDATA%/DreamerStudio/settings.json and persists across restarts
 AC-3. Invalid values are rejected with a clear message
-AC-4. Each section can be reset to default values</t>
+AC-4. Each section can be reset to default values after a confirmation; resetting Storage opens the default app data directory (REQ-008)</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2483,8 @@
         <is>
           <t>AC-1. User can switch language between VN and EN; the UI updates immediately
 AC-2. User can switch theme between light and dark; the UI updates immediately
-AC-3. On first launch, settings.json is created with the defaults: light theme and English</t>
+AC-3. On first launch, settings.json is created with the defaults: light theme and English
+AC-4. Language and theme changed anywhere (Settings or top bar) are saved and applied on the next start before the first screen shows</t>
         </is>
       </c>
     </row>
@@ -2506,12 +2506,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Let users change where application data is stored</t>
+          <t>Let users open another folder as the app data directory</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>In the Storage section, the user sees the current app data directory and can move it to another folder, with checks and a choice to move existing data or start empty. Moving covers database.sqlite, library, logs and cache; settings.json stays in place (TSK-010).</t>
+          <t>In the Storage section, the user sees the current app data directory and can open another folder instead. Data is not moved: a folder with Dreamer Studio data (database.sqlite) is opened as is; an empty folder gets new data. The switch applies without restarting. settings.json stays in place (TSK-010).</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -2527,10 +2527,11 @@
       <c r="H4" s="1" t="inlineStr">
         <is>
           <t>AC-1. Current app data directory is shown with a button to open it in Explorer
-AC-2. User can pick a new folder; the app checks write permission and free space first
-AC-3. User chooses to move existing data or start with an empty folder
-AC-4. Moving data shows progress; on failure the old directory stays in use and its data is untouched
-AC-5. Change is blocked while pipelines are running</t>
+AC-2. User can pick another folder; the app checks write permission first
+AC-3. A folder with Dreamer Studio data is opened as is (upgraded if older); a folder without it gets new empty data
+AC-4. The switch applies without restarting, behind a loading popup; on failure the app stays on the previous directory and shows why
+AC-5. Change is blocked while pipelines are queued or running
+AC-6. Data in the previous directory is never changed or deleted</t>
         </is>
       </c>
     </row>
@@ -2574,8 +2575,8 @@
         <is>
           <t>AC-1. Settings are read from %LOCALAPPDATA%/DreamerStudio/settings.json at startup
 AC-2. Missing file is created with default values; default app data directory is %LOCALAPPDATA%/DreamerStudio
-AC-3. Invalid or corrupted file falls back to default values, is logged, and the user is notified
-AC-4. If the configured app data directory is missing or unreachable, the app warns and lets the user pick another folder or use the default</t>
+AC-3. Invalid fields fall back to their defaults and valid fields are kept; an unreadable file falls back to all defaults and is kept as settings.json.bak; the problem is logged and the user is notified
+AC-4. If the configured app data directory does not exist or is not writable at startup, a dialog shows before anything else starts: pick another folder, use the default folder, or quit</t>
         </is>
       </c>
     </row>
@@ -2617,10 +2618,10 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can set max concurrent pipelines within an allowed range, with a default value
+          <t>AC-1. User can set max concurrent pipelines from 1 to 5; default 1
 AC-2. New value applies to queued pipelines without restarting the app
 AC-3. Lowering the value does not stop pipelines that are already running
-AC-4. Pipeline Executor (TSK-008) reads the concurrency limit from settings.json instead of the fixed value 1; default value is 1</t>
+AC-4. Pipeline Executor (TSK-008) uses this setting instead of the fixed value 1; default 1</t>
         </is>
       </c>
     </row>
@@ -2672,9 +2673,9 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Shows app name, version, build date, license, and repository link
+          <t>AC-1. Shows app name, version, build date ('dev' in dev mode), license (MIT), and repository link (opens in the browser)
 AC-2. Version comes from the single source of truth (TSK-002)
-AC-3. User can copy version info to the clipboard for bug reports</t>
+AC-3. User can copy version info (version, build date, Electron, Chromium, Node, Windows version) to the clipboard for bug reports</t>
         </is>
       </c>
     </row>
@@ -2716,10 +2717,11 @@
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Each check returns OK/Warning/Error, a message, and a suggested fix
+          <t>AC-1. Each check has a category and returns OK/Warning/Error, a message, and a suggested fix for Warning/Error, in the UI language
 AC-2. New checks can be registered without changing the engine
-AC-3. Built-in check: read &amp; write permission on the app data directory (default %LOCALAPPDATA%/DreamerStudio)
-AC-4. TODO: more checks will be defined once the architecture is ready (TSK-001)</t>
+AC-3. Built-in check: read &amp; write permission on the configured app data directory and the settings folder
+AC-4. Built-in checks also cover: database integrity, AI backend running and reachable, settings.json valid (Warning when defaults were used), free disk space on the app data drive (Warning below 1 GB)
+AC-5. A check that throws or times out returns Error; the other checks still run</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2763,7 @@
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can run all checks on demand; results are grouped by category
+          <t>AC-1. Checks run when the page opens and on demand; results are grouped by category, one list item per check with a status dot
 AC-2. Shows the results of all checks registered in the self-check engine (TSK-011)
 AC-3. Warning and Error results show the suggested fix</t>
         </is>
@@ -2790,7 +2792,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>Export a zip file containing the diagnostics results, app and system info, and recent logs.</t>
+          <t>Removed from release 0.0.0 by the human on 2026-10-20: diagnostics are stateless and show results directly; no report file. Kept as an idea. Previous scope: export one JSON file with the diagnostics results, app and system info, settings, and the last 500 lines of the main and backend logs.</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -2800,14 +2802,14 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>0. Idea</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Export creates a zip with diagnostics results, app/system info, and recent logs
+          <t>AC-1. Export creates one JSON file with diagnostics results, app/system info, settings, and the last 500 lines of the main and backend logs
 AC-2. User chooses where to save the file
-AC-3. Sensitive data (API keys, tokens) is never included</t>
+AC-3. Sensitive data (API keys, tokens, the Windows user name in paths) is partly masked with *, keeping the first and last characters for debugging</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(TSK010): Store application settings in a JSON file at a fixed location
- docs(settings): document the settings file [TSK-010]
- fix(settings): resolve review and test findings [TSK-010]
- feat(settings): ask for another app data folder at startup [TSK-010]
- feat(settings): store app settings in settings.json [TSK-010]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -2568,7 +2568,7 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -3931,7 +3931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5781,21 +5781,74 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n"/>
-      <c r="B37" s="1" t="n"/>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="1" t="n"/>
-      <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-      <c r="G37" s="1" t="n"/>
-      <c r="H37" s="1" t="n"/>
-      <c r="I37" s="1" t="n"/>
-      <c r="J37" s="1" t="n"/>
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>AD-36</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>How settings.json is validated</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>settings.json can be edited by hand or damaged; TSK-010 AC-3 needs each invalid field to fall back to its default while valid fields are kept. TH02-01 solution Q-01.</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>TH02-01, TSK-010, REQ-006</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Hand-written sanitizer in shared/ — four fields, no dependency, same code in main and renderer
+Schema library (zod / valibot) — Cons: new dependency for four fields; per-field fallback still hand-written</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>Hand-written sanitizer in shared/</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>Hand-written sanitizer in shared/</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-01 on 2026-10-20. Built in TSK-010: shared/models/settings.ts sanitizeSettings (invalid field names returned), electron/main/settings/settings-store.ts.</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="1" t="n"/>
+      <c r="C38" s="1" t="n"/>
+      <c r="D38" s="1" t="n"/>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+      <c r="J38" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REQ007,REQ009): Save language and theme from the top bar, run pipelines up to the max concurrent setting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -2476,7 +2476,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(REQ008): Let users open another app data folder without restarting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -3931,7 +3931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5834,21 +5834,74 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="1" t="n"/>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-      <c r="G38" s="1" t="n"/>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="1" t="n"/>
-      <c r="J38" s="1" t="n"/>
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>AD-37</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>How main code reaches the current app data after a live switch</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>REQ-008 switches the app data folder without a restart; IPC handlers, error handlers and the backend held AppPaths, the Database and the executor as values captured at startup. TH02-01 solution Q-02.</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>TH02-01, REQ-008, TSK-007, TSK-008</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Getter on one AppDataManager — handlers registered once, read the current session per call; while switching session() throws APP_DATA_SWITCHING
+Re-register handlers on every switch — Cons: ipcMain handlers removed and added at runtime, easy to leak listeners or miss one</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>Getter on one AppDataManager</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>Getter on one AppDataManager</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>Human answered Q-02 on 2026-10-19. Built in REQ-008: electron/main/app-data/app-data-manager.ts (current, session, paths), app-data-session.ts; app-ipc, pipeline-ipc and error-handlers take getters.</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="1" t="n"/>
+      <c r="C39" s="1" t="n"/>
+      <c r="D39" s="1" t="n"/>
+      <c r="E39" s="1" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="1" t="n"/>
+      <c r="I39" s="1" t="n"/>
+      <c r="J39" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
build: refactor the structure of the project
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -2343,7 +2343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2770,48 +2770,14 @@
       </c>
     </row>
     <row r="11" ht="52.8" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>REQ-012</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>TH-02 Configuration - Diagnostics &amp; About - Diagnostics &amp; About</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>Export Diagnostics Report</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Export a report to attach to bug reports</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>Removed from release 0.0.0 by the human on 2026-10-20: diagnostics are stateless and show results directly; no report file. Kept as an idea. Previous scope: export one JSON file with the diagnostics results, app and system info, settings, and the last 500 lines of the main and backend logs.</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>0.0.0</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="inlineStr">
-        <is>
-          <t>0. Idea</t>
-        </is>
-      </c>
-      <c r="H11" s="1" t="inlineStr">
-        <is>
-          <t>AC-1. Export creates one JSON file with diagnostics results, app/system info, settings, and the last 500 lines of the main and backend logs
-AC-2. User chooses where to save the file
-AC-3. Sensitive data (API keys, tokens, the Windows user name in paths) is partly masked with *, keeping the first and last characters for debugging</t>
-        </is>
-      </c>
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
@@ -3053,20 +3019,10 @@
       <c r="G35" s="1" t="n"/>
       <c r="H35" s="1" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="n"/>
-      <c r="B36" s="1" t="n"/>
-      <c r="C36" s="1" t="n"/>
-      <c r="D36" s="1" t="n"/>
-      <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="n"/>
-      <c r="G36" s="1" t="n"/>
-      <c r="H36" s="1" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REQ011): Show self-check results grouped by category in Settings › Diagnostics
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">

</xml_diff>

<commit_message>
chore(solu): prototype the library list screen in Storybook
- Story `Pages/Library` on the Main layout: left filter panel (search, sort, scope, source language, publication,
  app tags, genre), page toolbar with Novels / Musics / Videos tabs (Musics and Videos show coming soon),
  grid / list items and a right Novel inspector (stats, metadata with in-place edit, export, delete).
- Import states of a novel as story args, plus empty library, load error and novel page stories.
- `ds-pill` gets an opt-in `dot`; library styles in `_library-*.scss`, texts in i18n.
- Shell takes `initialRailExpanded`; the top bar shows "Novels" as the Library page name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>Shared local persistence layer for all features: a local database (pipeline history, and later library metadata) and a defined folder layout inside the app data directory (library, logs, cache). Includes schema migration so data survives upgrades between releases.</t>
+          <t>Shared local persistence layer for all features: a local database (pipeline runs, operations, and history; library data is stored in files, AD-38) and a defined folder layout inside the app data directory (library, logs, cache). Includes schema migration so data survives upgrades between releases.</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>Defines the Dreamer package format (.zip with metadata.json, an optional cover, and chapters/*.txt) and imports one package at a time from an Import screen. The package type comes from metadata.json (only novel in 0.1.0). The package is read and checked without writing anything, the user reviews and edits a preview, then the import runs as a background pipeline. Every import creates a new novel; there is no duplicate check and no import into an existing novel. Chapter content and cover are stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/, metadata and chapter list in SQLite. The same format is used by Export (TH03-02).</t>
+          <t>Defines the Dreamer package format (.zip with metadata.json, an optional cover, and chapters/*.txt) and imports one package at a time from an Import screen. The package type comes from metadata.json (only novel in 0.1.0). The package is read and checked without writing anything, the user reviews and edits a preview, then the import runs as a background pipeline. Every import creates a new novel; there is no duplicate check and no import into an existing novel. Each novel is stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/: metadata.json (metadata and chapter list), cover, and chapter text; nothing of the library is stored in SQLite (TSK-013, AD-38). The same format is used by Export (TH03-02).</t>
         </is>
       </c>
       <c r="G10" s="1" t="inlineStr">
@@ -814,7 +814,7 @@
 2. Import screen opened from Home and Library: pick or drop one package, check it, preview and edit, then import as a background pipeline
 3. invalid package rejected with a clear list of problems; nothing written
 4. every import creates a new novel (no duplicate check, no import into an existing novel)
-5. chapter content and cover stored as files in &lt;app data&gt;/library, metadata in SQLite</t>
+5. each novel stored as files in &lt;app data&gt;/library: metadata.json with metadata and chapter list, cover, and chapter files</t>
         </is>
       </c>
     </row>
@@ -846,15 +846,15 @@
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>Library screen listing all imported novels with search, filter, and sort, and a novel detail page. The user can edit a novel's metadata (title, author, cover, tags, description), manage its chapters (rename, reorder, merge, split, delete), delete novels, and export a novel to a Dreamer package.</t>
+          <t>Library screen listing all imported novels in a grid or list, with a Filters panel (search, sort, language, publication status, genre) and an inspector for the active novel. From the inspector the user edits a novel's metadata (title, author, cover, tags, description, publication status), deletes novels, exports a novel to a Dreamer package, opens its folder, and opens its detail page (TH03-03). Analysed / Translated counts and filters and the Musics / Videos tabs are shown as "Coming soon" (TH04 or later).</t>
         </is>
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>1. library screen lists novels with search, filter, and sort
-2. edit novel metadata (title, author, cover, tags, description)
-3. chapter management (rename, reorder, merge, split, delete)
-4. delete novels with all their data
+          <t>1. library screen lists novels in a grid or list with search, filters (language, publication status, genre), and sort
+2. inspector for the active novel with its stats, metadata, and actions
+3. edit novel metadata (title, author, cover, tags, description, publication status)
+4. delete one or many novels with all their data
 5. export a novel to a Dreamer package that can be re-imported</t>
         </is>
       </c>
@@ -867,12 +867,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>Read novel chapters inside the app</t>
+          <t>Read and organize a novel's chapters inside the app</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -887,14 +887,17 @@
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>Reader screen to read a novel chapter by chapter, with a table of contents, next/previous navigation, and keyboard shortcuts. Reading settings (font, font size, line height, content width) apply to all novels. The user can search text across the novel's chapters. No bookmarks and no auto resume in 0.1.0.</t>
+          <t>Novel detail page opened from the library screen, built as a reader: Chapters panel on the left (table of contents, search, Organize mode), chapter reader in the center, and Reading / Search tabs on the right. The user reads chapter by chapter with next/previous navigation, keyboard shortcuts, and a Focus mode; manages chapters (rename, reorder, merge, split, delete); edits the current chapter's title and text; changes reading settings (font, font size, line height, content width) that apply to all novels; and searches text across the novel's chapters. No bookmarks and no auto resume in 0.1.0.</t>
         </is>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>1. table of contents and chapter navigation (next/previous, keyboard shortcuts)
-2. reading settings (font, font size, line height, content width) applied to all novels
-3. search text across the novel's chapters</t>
+          <t>1. novel detail page with Chapters panel, reader, and Reading / Search tabs
+2. chapter navigation (next/previous, keyboard shortcuts) and Focus mode
+3. chapter management (rename, reorder, merge, split, delete)
+4. edit the current chapter's title and text
+5. reading settings (font, font size, line height, content width) applied to all novels
+6. search text across the novel's chapters</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3129,7 +3132,7 @@
       <c r="H2" s="1" t="inlineStr">
         <is>
           <t>AC-1. Spec in _docs defines the zip layout: metadata.json at the root, optional cover image (JPG/PNG), and chapter files in chapters/
-AC-2. metadata.json fields are defined with type and required/optional: format version, package type, original title, title, author, description, tags, language (BCP-47, required), cover file, and the ordered chapter list (file, title)
+AC-2. metadata.json fields are defined with type and required/optional: format version, package type, original title, title, author, description, tags, language (BCP-47, required), publication ('ongoing' | 'completed', optional), cover file, and the ordered chapter list (file, title)
 AC-3. A package type other than novel is rejected as not supported yet
 AC-4. The format has a version number; packages with an unsupported version are rejected
 AC-5. Chapter files are UTF-8 plain text; a file that is not valid UTF-8 rejects the package with a reason naming the file; a BOM is removed and line endings are normalized on import
@@ -3137,7 +3140,8 @@
 AC-7. Spec lists the size limits (zip size, unpacked size, entry count, cover size), and each limit is checked
 AC-8. Entries with unsafe paths (absolute, drive letter, "..") or duplicate names, a chapter file listed twice, and a listed file that is missing reject the package; entries not listed in metadata.json are ignored and shown in the preview
 AC-9. Spec defines one paragraph rule (blank and whitespace-only lines, line breaks inside a paragraph, trimming), used by import, export, chapter split, reader, and search
-AC-10. Spec includes a sample package that is also used by tests</t>
+AC-10. Spec includes a sample package that is also used by tests
+AC-11. A package without publication imports as 'ongoing'</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3163,12 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Store imported novels on disk and in the database</t>
+          <t>Store imported novels in the file system</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Chapter content and cover are stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/. Metadata, tags, and the chapter list are stored in SQLite through the shared data access layer (TSK-005); library tables are added by a schema migration (TSK-006). Internal IDs keep file names stable and prepare per-chapter translations (TH04-05).</t>
+          <t>Each novel is stored in &lt;app data&gt;/library/&lt;novel-uuid&gt;/: metadata.json (novel metadata and the ordered chapter list), the cover, and chapters/&lt;content-hash&gt;.txt. metadata.json is written atomically. SQLite keeps only operations and history (pipeline runs, logs), no library data (AD-38).</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -3179,15 +3183,17 @@
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Chapter content and cover are stored in &lt;app data&gt;/library/&lt;novel-uuid&gt;/
-AC-2. Novel metadata (original title, title, author, description, language, import date), tags, and chapter list (order, title, file) are stored in SQLite through the shared data access layer (TSK-005)
-AC-3. Library tables are created by a schema migration (TSK-006)
-AC-4. Deleting a novel removes its database rows and its folder
-AC-5. Self-check (TSK-011) reports novels whose files are missing and library folders with no novel
-AC-6. Each novel and chapter has an internal ID; chapter files are named by chapter ID, so reordering never renames files
-AC-7. Folder and file names use internal IDs only, never values from the package
-AC-8. Each chapter stores a content hash and paragraph count
-AC-9. Leftovers of an interrupted import (staging folders, folders with no novel) are removed at startup</t>
+          <t>AC-1. Each novel is stored in &lt;app data&gt;/library/&lt;novel-uuid&gt;/ with metadata.json, an optional cover.jpg or cover.png, and chapter files in chapters/
+AC-2. metadata.json has a format version and holds the novel metadata (original title, title, author, description, language, tags, publication), the import date, the updated date, and the ordered chapter list
+AC-3. Each chapter entry has title, file, content hash, paragraph count, and character count
+AC-4. Chapter files are named by their content hash (chapters/&lt;content-hash&gt;.txt); reorder and rename only rewrite metadata.json
+AC-5. Merge, split, and edit write the new chapter files first, then update metadata.json; chapter files no longer referenced are removed
+AC-6. metadata.json is written atomically (temp file, then rename), so it is never left half written
+AC-7. No library data is stored in SQLite; SQLite keeps only operations and history (AD-38)
+AC-8. Deleting a novel removes its folder
+AC-9. Folder and file names use internal IDs or content hashes only, never values from the package
+AC-10. Self-check (TSK-011) reports files referenced by metadata.json that are missing, and library folders without a valid metadata.json
+AC-11. Leftovers are removed at startup: staging folders of an interrupted import, temp files, and unreferenced chapter files</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3242,7 @@
 AC-5. User can untick chapters and edit chapter titles before the import
 AC-6. Import starts a pipeline run that appears in the pipeline monitor and history (REQ-004, REQ-005); the user can leave the screen while it runs
 AC-7. A failed, cancelled, or interrupted import (app closed or crashed) leaves no partial novel in the library
-AC-8. The Library screen (REQ-014) shows running imports in a separate section, and the novel appears when the import succeeds
+AC-8. A novel being imported is shown in the Library screen list (REQ-014) with its import progress and cannot be opened until the import finishes
 AC-9. When an import finishes, one notification per package shows the result, with an action to open the novel on success
 AC-10. Every import creates a new novel, even when the same package was imported before</t>
         </is>
@@ -3275,7 +3281,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Library screen opened from the sidebar, listing all novels with search, filter, and sort. Opening a novel shows its detail page (REQ-023).</t>
+          <t>Library screen opened from the sidebar. Toolbar with media tabs, novel count, Grid / List view, and "Import package" (REQ-013); Filters panel on the left, grid or list of novels in the center, inspector for the active novel on the right. Opening a novel shows its detail page (REQ-023). Analysed / Translated data and the Musics / Videos tabs come in TH04 or later.</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -3291,14 +3297,20 @@
       <c r="H6" s="1" t="inlineStr">
         <is>
           <t>AC-1. Library item in the sidebar is enabled (no longer "Coming soon") and opens the library screen
-AC-2. Each novel shows its cover (or a placeholder), title, author, chapter count, and tags
-AC-3. User can search novels by title or author
-AC-4. User can filter novels by tag
-AC-5. User can sort novels by title, author, or import date, ascending or descending
-AC-6. Empty library shows an empty state with an "Import package" action
-AC-7. A search or filter with no match shows a no-results state with a "Clear filters" action
-AC-8. User can select several novels for a bulk action (delete, REQ-017)
-AC-9. Opening a novel shows its detail page (REQ-023)</t>
+AC-2. Toolbar shows the Novels tab, the novel count, a Grid / List view switch, and an "Import package" action; the Musics and Videos tabs show "Coming soon"
+AC-3. Each novel shows its cover (or a placeholder), title, author, chapter count, and tags
+AC-4. User can search novels by title, original title, or author; "/" focuses the search field, except while typing in a field
+AC-5. User can filter novels by source language, publication status (ongoing / completed), and genre (the novel's tags); several selected genres combine with AND
+AC-6. User can sort novels by title, author, import date, last updated, or chapter count, ascending or descending
+AC-7. Analysed / Translated filters and counts and the app tags filter show "Coming soon"
+AC-8. Clicking a novel makes it the active novel; the inspector shows its cover, title, author · language · publication status, stats (chapters, characters; analysed and translated "Coming soon"), and metadata
+AC-9. Inspector has the actions Open, Export (REQ-018), Change cover, Remove cover (REQ-015), Open folder, Delete (REQ-017), and Edit for the metadata (REQ-015)
+AC-10. Open folder shows the novel's folder in the system file manager
+AC-11. Double-click, Enter, or Open shows the novel's detail page (REQ-023)
+AC-12. User can select several novels for a bulk action (delete, REQ-017)
+AC-13. Empty library shows an empty state with an "Import package" action
+AC-14. A search or filter with no match shows a no-results state with a "Clear filters" action
+AC-15. A novel being imported is shown in the list with its import progress and cannot be opened until the import succeeds (REQ-013 AC-8)</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3337,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>From the novel detail page, the user edits the title, author, description, tags, and cover.</t>
+          <t>In the inspector of the library screen (REQ-014), the user edits the title, original title, language, author, publication status, description, tags, and cover of the active novel.</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -3340,18 +3352,18 @@
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can edit title, author, description, and tags from the novel detail page and save or cancel the changes
+          <t>AC-1. User can edit title, original title, language, author, publication status (ongoing / completed), description, and tags in the inspector and save or cancel the changes
 AC-2. User can replace the cover with a JPG/PNG image or remove it
-AC-3. Title is required; invalid values (e.g. a cover that is too large or not an image) are rejected with a clear message
-AC-4. Leaving the page with unsaved changes asks for confirmation
-AC-5. Changes are shown in the library screen immediately</t>
+AC-3. Title, original title, and language are required; invalid values (e.g. a cover that is too large or not an image) are rejected with a clear message
+AC-4. Leaving the edit with unsaved changes (another novel or another page) asks for confirmation
+AC-5. Changes are shown in the library list and the inspector immediately</t>
         </is>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>REQ-016</t>
+          <t>REQ-017</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -3361,17 +3373,17 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Chapter Management</t>
+          <t>Delete Novel</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>Let users organize the chapters of a novel</t>
+          <t>Let users remove novels from the library</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>From the chapter list of the novel detail page, the user renames, reorders, merges, splits, and deletes chapters.</t>
+          <t>The user deletes the active novel from the inspector of the library screen (REQ-014), or many novels with multi-select. A bulk delete skips locked novels (TSK-024).</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
@@ -3386,19 +3398,16 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can rename a chapter
-AC-2. User can reorder chapters by drag and drop or with the keyboard
-AC-3. User can merge two or more consecutive chapters into one; the merged chapter keeps the title of the first
-AC-4. User can split a chapter into two at a chosen paragraph, with a preview of the paragraphs
-AC-5. User can delete one or many chapters after confirmation
-AC-6. A failed merge or split leaves the chapters unchanged</t>
+          <t>AC-1. User can delete one or many novels after a confirmation that names the novel, or says how many novels will be deleted
+AC-2. All data of the novel is deleted: files, metadata, and chapters
+AC-3. A novel cannot be deleted while a pipeline (e.g. export) is running on it (TSK-024); a bulk delete skips locked novels and the confirmation names the skipped ones</t>
         </is>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>REQ-017</t>
+          <t>REQ-018</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3408,17 +3417,17 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Delete Novel</t>
+          <t>Export Novel Package</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>Let users remove novels from the library</t>
+          <t>Let users export a novel to a Dreamer package</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>The user deletes one or many novels from the library screen or the novel detail page.</t>
+          <t>From the inspector of the library screen (REQ-014), the user exports the novel to a Dreamer package (.zip) for backup or sharing. Export runs as a background pipeline.</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
@@ -3433,17 +3442,19 @@
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can delete one or many novels after a confirmation that names the novel or the count
-AC-2. All data of the novel is deleted: files, metadata, and chapters
-AC-3. A novel cannot be deleted while a pipeline (e.g. export) is running on it (TSK-024)
-AC-4. Deleting from the detail page returns to the library screen</t>
+          <t>AC-1. User can export a novel from the library screen inspector and choose where to save the .zip; the default file name is the novel title
+AC-2. Export runs as a pipeline run and appears in the pipeline monitor and history
+AC-3. The exported package follows the format spec (TSK-012) with the current metadata, cover, and chapters in their current order
+AC-4. Importing the exported package into an empty library gives the same metadata (including publication status) and chapters (round trip)
+AC-5. A failed or cancelled export leaves no partial .zip file
+AC-6. When the export finishes, a notification offers to show the file in its folder</t>
         </is>
       </c>
     </row>
     <row r="10" ht="118.8" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>REQ-018</t>
+          <t>TSK-024</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -3453,17 +3464,17 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Export Novel Package</t>
+          <t>Novel Pipeline Lock</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Let users export a novel to a Dreamer package</t>
+          <t>Keep a novel consistent while a pipeline works on it</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>From the novel detail page, the user exports the novel to a Dreamer package (.zip) for backup or sharing. Export runs as a background pipeline.</t>
+          <t>Pipeline runs record which novel they work on (TSK-008). While a run on a novel is queued or running, the novel is locked: no metadata edit (REQ-015), chapter change (REQ-016), chapter edit (REQ-026), or delete (REQ-017).</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
@@ -3478,19 +3489,17 @@
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can export a novel from its detail page and choose where to save the .zip; the default file name is the novel title
-AC-2. Export runs as a pipeline run and appears in the pipeline monitor and history
-AC-3. The exported package follows the format spec (TSK-012) with the current metadata, cover, and chapters in their current order
-AC-4. Importing the exported package into an empty library gives the same metadata and chapters (round trip)
-AC-5. A failed or cancelled export leaves no partial .zip file
-AC-6. When the export finishes, a notification offers to show the file in its folder</t>
+          <t>AC-1. Each pipeline run on a novel records the novel's ID
+AC-2. While a run on a novel is queued or running, edit, chapter change, chapter edit, and delete of that novel are refused with a clear reason
+AC-3. The lock is released when the run succeeds, fails, or is cancelled, and after an app restart
+AC-4. Reading and searching a locked novel still work</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>REQ-023</t>
+          <t>TSK-025</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3500,17 +3509,17 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>Novel Detail Page</t>
+          <t>Library File Access for the UI</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>Show one novel and give access to all its actions</t>
+          <t>Let the UI show covers and chapter text stored in the library</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>Page opened from the library screen (REQ-014). Shows the novel's metadata and chapter list, and is the entry point for reading (REQ-019), editing (REQ-015), chapter management (REQ-016), export (REQ-018), and delete (REQ-017).</t>
+          <t>The renderer cannot read files directly (AD-06). Main serves library files (covers, chapter text) to the renderer in a safe way, limited to &lt;app data&gt;/library, and a preview of a cover image the user just picked, before save.</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -3525,83 +3534,46 @@
       </c>
       <c r="H11" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Page shows cover, title, author, description, tags, language, chapter count, and import date
-AC-2. Page lists all chapters in order; selecting a chapter opens it in the reader
-AC-3. Page has Read, Edit, Export, and Delete actions
-AC-4. Page shows loading, error, and not-found states
-AC-5. Page shows when a pipeline is running on the novel, and actions blocked by it are disabled with the reason (TSK-024)</t>
+          <t>AC-1. The UI can show a novel's cover, a preview of a cover image the user just picked (before save), and load a chapter's text, without the renderer reading files outside &lt;app data&gt;/library
+AC-2. Only files inside &lt;app data&gt;/library can be read; other paths are refused
+AC-3. The page security policy is not weakened to allow other file access</t>
         </is>
       </c>
     </row>
     <row r="12" ht="105.6" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>TSK-024</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>Novel Pipeline Lock</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Keep a novel consistent while a pipeline works on it</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>Pipeline runs record which novel they work on (TSK-008). While a run on a novel is queued or running, the novel is locked: no metadata edit (REQ-015), chapter change (REQ-016), or delete (REQ-017).</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="inlineStr">
-        <is>
-          <t>2. Approve</t>
-        </is>
-      </c>
-      <c r="H12" s="1" t="inlineStr">
-        <is>
-          <t>AC-1. Each pipeline run on a novel records the novel's ID
-AC-2. While a run on a novel is queued or running, edit, chapter change, and delete of that novel are refused with a clear reason
-AC-3. The lock is released when the run succeeds, fails, or is cancelled, and after an app restart
-AC-4. Reading and searching a locked novel still work</t>
-        </is>
-      </c>
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
     </row>
     <row r="13" ht="79.2" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>TSK-025</t>
+          <t>REQ-019</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>Library File Access for the UI</t>
+          <t>Novel Reader</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Let the UI show covers and chapter text stored in the library</t>
+          <t>Let users read a novel chapter by chapter</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>The renderer cannot read files directly (AD-06). Main serves library files (covers, chapter text) to the renderer in a safe way, limited to &lt;app data&gt;/library.</t>
+          <t>Reader in the center of the novel detail page (REQ-023); the Chapters panel is the table of contents. Next/previous navigation, keyboard shortcuts, and a Focus mode.</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
@@ -3616,109 +3588,56 @@
       </c>
       <c r="H13" s="1" t="inlineStr">
         <is>
-          <t>AC-1. The UI can show a novel's cover and load a chapter's text
-AC-2. Only files inside &lt;app data&gt;/library can be read; other paths are refused
-AC-3. The page security policy is not weakened to allow other file access</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="79.2" customHeight="1">
-      <c r="A14" s="1" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="1" t="n"/>
-      <c r="D14" s="1" t="n"/>
-      <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="n"/>
-      <c r="G14" s="1" t="n"/>
-      <c r="H14" s="1" t="n"/>
-    </row>
-    <row r="15" ht="66" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>REQ-019</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>Novel Reader</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Let users read a novel chapter by chapter</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>Reader screen opened from the novel detail page, with a table of contents, next/previous navigation, and keyboard shortcuts.</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="G15" s="1" t="inlineStr">
-        <is>
-          <t>2. Approve</t>
-        </is>
-      </c>
-      <c r="H15" s="1" t="inlineStr">
-        <is>
-          <t>AC-1. User can open the reader from the novel detail page or from a chapter in the chapter list
-AC-2. Table of contents lists all chapters and shows the current one; selecting a chapter opens it
-AC-3. User can go to the next/previous chapter with buttons and keyboard shortcuts; they are disabled on the first/last chapter, and shortcuts do not fire while typing in a field
+          <t>AC-1. Opening a novel shows its first chapter in the reader (no auto resume in 0.1.0)
+AC-2. The Chapters panel is the table of contents: it lists all chapters and marks the current one; selecting a chapter opens it
+AC-3. User can go to the next/previous chapter with buttons at the end of the chapter and with Alt+← / Alt+→; they are disabled on the first/last chapter, and shortcuts do not fire while typing in a field
 AC-4. Each paragraph of the plain-text chapter is shown as a separate paragraph
 AC-5. Reader colors follow the app theme (light/dark)
 AC-6. Reader shows the chapter position (e.g. "Chapter 12 / 340")
-AC-7. A chapter whose file is missing shows an error state instead of failing</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+AC-7. A chapter whose file is missing shows an error state with a "Try again" action instead of failing
+AC-8. User can enter Focus mode with the Focus button or Shift+F (not while typing) to hide the side panels, and leave it with the Focus button or Esc</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="79.2" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>REQ-020</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Reading Settings</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Let users adjust how chapter text is displayed</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>From the reader, the user changes the font, font size, line height, and content width. Settings apply to all novels and are saved in settings.json.</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>In the Reading tab of the novel detail page (REQ-023), the user changes the font, font size, line height, and content width. Settings apply to all novels and are saved in settings.json.</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G16" s="1" t="inlineStr">
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H16" s="1" t="inlineStr">
-        <is>
-          <t>AC-1. User can change font, font size, line height, and content width from the reader
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. User can change font, font size, line height, and content width in the Reading tab
 AC-2. Changes apply immediately to the open chapter
 AC-3. Settings apply to all novels and persist across restarts in settings.json (TSK-010)
 AC-4. User can reset reading settings to default values
@@ -3726,61 +3645,197 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="15" ht="66" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>REQ-022</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Search in Novel</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Let users find text across the chapters of a novel</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>In the reader, the user searches text in all chapters of the open novel and jumps to a result.</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>In the Search tab of the novel detail page (REQ-023), the user searches text in all chapters of the novel and jumps to a result.</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G17" s="1" t="inlineStr">
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="H15" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can search text across all chapters of the open novel
 AC-2. Search is case-insensitive
 AC-3. Results are grouped by chapter, show a snippet with the match highlighted, and show the total count
 AC-4. Selecting a result opens the chapter at the match and keeps it highlighted
-AC-5. Search shows searching and no-results states; a new query cancels the previous one</t>
+AC-5. Search shows searching and no-results states; a new query cancels the previous one
+AC-6. Ctrl+Shift+F opens the Search tab and focuses the search field</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>REQ-023</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Novel Detail Page</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Show one novel as a reader with its chapters</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Page opened from the library screen (REQ-014), with a reader layout: Chapters panel on the left (chapter list, search, Organize mode of REQ-016), chapter reader in the center (REQ-019), and a right panel with the Reading (REQ-020) and Search (REQ-022) tabs. Metadata, export, and delete stay in the library screen.</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. Top bar breadcrumb shows "Library · Novels · &lt;novel title&gt;"
+AC-2. Page header shows the current chapter (e.g. "0012 · &lt;chapter title&gt;") and only two actions: Edit (REQ-026) and Focus (REQ-019)
+AC-3. Chapters panel lists all chapters in order; selecting a chapter opens it in the reader, except in Organize mode (REQ-016)
+AC-4. Chapters panel search: digits search by chapter number and Enter opens that chapter; text filters the list by chapter title
+AC-5. Right panel has the Reading (REQ-020) and Search (REQ-022) tabs
+AC-6. Page shows loading, error, and not-found states
+AC-7. Page shows a banner when a pipeline is running on the novel; Edit is disabled with the reason (TSK-024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>REQ-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Chapter Management</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Let users organize the chapters of a novel</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>In the Organize mode of the Chapters panel on the novel detail page (REQ-023), the user renames, reorders, merges, splits, and deletes chapters. Each change is saved at once.</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. User can rename a chapter
+AC-2. User can reorder chapters by drag and drop or with the keyboard
+AC-3. User can merge two or more consecutive chapters into one; the merged chapter keeps the title of the first
+AC-4. User can split a chapter of at least 2 paragraphs into two at a chosen paragraph, with a preview of the paragraphs; the new second chapter gets the default title "{title} (2)", which the user can change
+AC-5. User can delete one or many chapters after confirmation
+AC-6. A failed merge, split, reorder, or delete leaves the chapters unchanged
+AC-7. Chapter changes are made in an Organize mode of the chapter list; each change is saved at once
+AC-8. A chapter title cannot be empty; rename or split with an empty title is refused</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n"/>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
-      <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="n"/>
-      <c r="G18" s="1" t="n"/>
-      <c r="H18" s="1" t="n"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>REQ-026</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>Edit Chapter</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Let users fix the title and text of a chapter</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Edit in the header of the novel detail page (REQ-023) opens an editor for the current chapter's title and text in place of the reader (REQ-019). Refused while the novel is locked (TSK-024).</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. Edit opens an editor for the current chapter's title and text in place of the reader; the text shows one paragraph per line
+AC-2. Editor has Save and Cancel; Save is disabled until something changes
+AC-3. Title and text are required; saving an empty title or text is refused with a clear message
+AC-4. After save, the reader shows the new title and text, and the chapter's character and paragraph counts are updated
+AC-5. Cancelling or leaving the page with unsaved changes asks for confirmation
+AC-6. The Chapters panel and the Search tab are disabled while editing
+AC-7. Edit is refused while the novel is locked (TSK-024)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -3982,10 +4037,20 @@
       <c r="G38" s="1" t="n"/>
       <c r="H38" s="1" t="n"/>
     </row>
+    <row r="39">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="1" t="n"/>
+      <c r="C39" s="1" t="n"/>
+      <c r="D39" s="1" t="n"/>
+      <c r="E39" s="1" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="1" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
     </dataValidation>
   </dataValidations>
@@ -3999,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4183,7 +4248,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Local database for pipeline history, library metadata, bookmarks.
+          <t>Local database for pipeline runs, operations, and history; library data is stored in files (AD-38).
 Risk (resolved 2026-10-17): node:sqlite is experimental in Node; require('node:sqlite') was broken in some Electron releases (fixed in 36.7.3 / 37.2.3 / 38). Electron is pinned to 44.9.0 and the TSK-002 spike proves it.</t>
         </is>
       </c>
@@ -5955,21 +6020,74 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
-      <c r="G39" s="1" t="n"/>
-      <c r="H39" s="1" t="n"/>
-      <c r="I39" s="1" t="n"/>
-      <c r="J39" s="1" t="n"/>
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>AD-38</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>Library storage</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>Where the library data (novel metadata, tags, publication, dates, chapter list) is stored. The previous TH03-01 design kept it in SQLite tables, with only chapter text and cover in files.</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>TSK-013, TH03-01, TH03-02, TH03-03, TSK-024</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>Files: metadata.json per novel — library data in the file system, SQLite only for operations and history
+SQLite tables — novel, novel_tag, chapter rows (previous TH03-01 design)</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>Files: metadata.json per novel</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>Files: metadata.json per novel</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>Human decision in the TH03-02 / TH03-03 solution review</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n"/>
+      <c r="B40" s="1" t="n"/>
+      <c r="C40" s="1" t="n"/>
+      <c r="D40" s="1" t="n"/>
+      <c r="E40" s="1" t="n"/>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="n"/>
+      <c r="H40" s="1" t="n"/>
+      <c r="I40" s="1" t="n"/>
+      <c r="J40" s="1" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided,Deferred"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(solu): define solution and prototype for importing novel
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -800,20 +800,20 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>Defines the Dreamer package format (.zip with metadata.json, an optional cover, and one plain-text file per chapter) and imports packages into the library as background pipelines. A package is validated before any data is written; a package whose ID already exists in the library is rejected. Chapter content and cover are stored as files in &lt;app data&gt;/library/&lt;novel-id&gt;/, metadata and chapter list in SQLite. The same format is used by Export (TH03-02).</t>
+          <t>Defines the Dreamer package format (.zip with metadata.json, an optional cover, and chapters/*.txt) and imports one package at a time from an Import screen. The package type comes from metadata.json (only novel in 0.1.0). The package is read and checked without writing anything, the user reviews and edits a preview, then the import runs as a background pipeline. Every import creates a new novel; there is no duplicate check and no import into an existing novel. Chapter content and cover are stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/, metadata and chapter list in SQLite. The same format is used by Export (TH03-02).</t>
         </is>
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
           <t>1. Dreamer package format (.zip) defined, versioned, and documented in _docs
-2. import one or more packages, each as a background pipeline
-3. package validated before import; invalid package rejected with a clear reason
-4. package with an ID that already exists in the library is rejected
+2. Import screen opened from Home and Library: pick or drop one package, check it, preview and edit, then import as a background pipeline
+3. invalid package rejected with a clear list of problems; nothing written
+4. every import creates a new novel (no duplicate check, no import into an existing novel)
 5. chapter content and cover stored as files in &lt;app data&gt;/library, metadata in SQLite</t>
         </is>
       </c>
@@ -841,7 +841,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -882,20 +882,19 @@
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>Reader screen to read a novel chapter by chapter, with a table of contents, next/previous navigation, and keyboard shortcuts. Reading settings (font, font size, line height, content width) apply to all novels. The user can bookmark positions and search text across the novel's chapters.</t>
+          <t>Reader screen to read a novel chapter by chapter, with a table of contents, next/previous navigation, and keyboard shortcuts. Reading settings (font, font size, line height, content width) apply to all novels. The user can search text across the novel's chapters. No bookmarks and no auto resume in 0.1.0.</t>
         </is>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
           <t>1. table of contents and chapter navigation (next/previous, keyboard shortcuts)
 2. reading settings (font, font size, line height, content width) applied to all novels
-3. bookmarks
-4. search text across the novel's chapters</t>
+3. search text across the novel's chapters</t>
         </is>
       </c>
     </row>
@@ -989,7 +988,7 @@
     <row r="16" ht="26.4" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>TH03-05</t>
+          <t>TH03-04</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1014,7 +1013,7 @@
     <row r="17" ht="26.4" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>TH03-06</t>
+          <t>TH03-05</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1039,7 +1038,7 @@
     <row r="18" ht="26.4" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>TH03-07</t>
+          <t>TH03-06</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1064,7 +1063,7 @@
     <row r="19" ht="26.4" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>TH03-08</t>
+          <t>TH03-07</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1089,7 +1088,7 @@
     <row r="20" ht="26.4" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>TH03-09</t>
+          <t>TH03-08</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -3036,7 +3035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3114,7 +3113,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Specification of the Dreamer package (.zip): metadata.json, an optional cover image, and one UTF-8 plain-text file per chapter. Documented in _docs and used by import (REQ-013) and export (REQ-018).</t>
+          <t>Specification of the Dreamer package (.zip): metadata.json, an optional cover image, and one UTF-8 plain-text file per chapter in chapters/. metadata.json names the package type, so the app knows what it imports without asking. Documented in _docs and used by import (REQ-013) and export (REQ-018).</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -3124,16 +3123,21 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Spec in _docs defines the zip layout: metadata.json, optional cover image (JPG/PNG), and one plain-text file per chapter
-AC-2. metadata.json fields are defined with type and required/optional: format version, package ID, title, author, description, tags, language, and the ordered chapter list (file, title)
-AC-3. Chapter files are UTF-8 plain text; paragraphs are separated by a blank line
+          <t>AC-1. Spec in _docs defines the zip layout: metadata.json at the root, optional cover image (JPG/PNG), and chapter files in chapters/
+AC-2. metadata.json fields are defined with type and required/optional: format version, package type, original title, title, author, description, tags, language (BCP-47, required), cover file, and the ordered chapter list (file, title)
+AC-3. A package type other than novel is rejected as not supported yet
 AC-4. The format has a version number; packages with an unsupported version are rejected
-AC-5. Spec includes a sample package that is also used by tests</t>
+AC-5. Chapter files are UTF-8 plain text; a file that is not valid UTF-8 rejects the package with a reason naming the file; a BOM is removed and line endings are normalized on import
+AC-6. A package with no chapters and an empty chapter file are both valid
+AC-7. Spec lists the size limits (zip size, unpacked size, entry count, cover size), and each limit is checked
+AC-8. Entries with unsafe paths (absolute, drive letter, "..") or duplicate names, a chapter file listed twice, and a listed file that is missing reject the package; entries not listed in metadata.json are ignored and shown in the preview
+AC-9. Spec defines one paragraph rule (blank and whitespace-only lines, line breaks inside a paragraph, trimming), used by import, export, chapter split, reader, and search
+AC-10. Spec includes a sample package that is also used by tests</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3164,7 @@
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>Chapter content and cover are stored as files in &lt;app data&gt;/library/&lt;novel-id&gt;/. Metadata, tags, and the chapter list are stored in SQLite through the shared data access layer (TSK-005); library tables are added by a schema migration (TSK-006).</t>
+          <t>Chapter content and cover are stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/. Metadata, tags, and the chapter list are stored in SQLite through the shared data access layer (TSK-005); library tables are added by a schema migration (TSK-006). Internal IDs keep file names stable and prepare per-chapter translations (TH04-05).</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -3170,16 +3174,20 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Chapter content and cover are stored in &lt;app data&gt;/library/&lt;novel-id&gt;/
-AC-2. Novel metadata, tags, and chapter list (order, title, file) are stored in SQLite through the shared data access layer (TSK-005)
+          <t>AC-1. Chapter content and cover are stored in &lt;app data&gt;/library/&lt;novel-uuid&gt;/
+AC-2. Novel metadata (original title, title, author, description, language, import date), tags, and chapter list (order, title, file) are stored in SQLite through the shared data access layer (TSK-005)
 AC-3. Library tables are created by a schema migration (TSK-006)
 AC-4. Deleting a novel removes its database rows and its folder
-AC-5. Self-check (TSK-011) reports novels whose files are missing</t>
+AC-5. Self-check (TSK-011) reports novels whose files are missing and library folders with no novel
+AC-6. Each novel and chapter has an internal ID; chapter files are named by chapter ID, so reordering never renames files
+AC-7. Folder and file names use internal IDs only, never values from the package
+AC-8. Each chapter stores a content hash and paragraph count
+AC-9. Leftovers of an interrupted import (staging folders, folders with no novel) are removed at startup</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3214,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>From the Library screen, the user picks one or more .zip packages. Each package is validated and imported as a background pipeline (TSK-008) that the user can follow in the pipeline monitor.</t>
+          <t>Import screen opened from Home and from the Library screen. The user picks or drops one .zip package; the app reads and checks it without writing anything and shows a preview. The user edits the metadata and the chapter list, then starts the import, which runs as a background pipeline (TSK-008).</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -3216,17 +3224,21 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can pick one or more .zip packages from the Library screen
-AC-2. Each package is imported as its own pipeline run and appears in the pipeline monitor and history (REQ-004, REQ-005)
-AC-3. The package is validated against the format spec (TSK-012) before any data is written; an invalid package fails with a clear reason (e.g. missing metadata.json, missing chapter file, unsupported version)
-AC-4. A package whose ID already exists in the library is rejected with a message naming the existing novel
-AC-5. A failed or cancelled import leaves no partial novel in the library
-AC-6. The novel appears in the library when the import succeeds</t>
+          <t>AC-1. User opens the Import screen from an Import button on Home or on the Library screen
+AC-2. User picks one .zip package or drops it on the screen; another file type is refused with a clear message
+AC-3. The package is read and checked against the format spec (TSK-012) without writing anything; an invalid package shows the list of problems and can be replaced by another file
+AC-4. The preview shows the metadata in a form the user can edit (title and language required) and the chapter list with checks (e.g. empty chapter, same text as another chapter, ignored files)
+AC-5. User can untick chapters and edit chapter titles before the import
+AC-6. Import starts a pipeline run that appears in the pipeline monitor and history (REQ-004, REQ-005); the user can leave the screen while it runs
+AC-7. A failed, cancelled, or interrupted import (app closed or crashed) leaves no partial novel in the library
+AC-8. The Library screen (REQ-014) shows running imports in a separate section, and the novel appears when the import succeeds
+AC-9. When an import finishes, one notification per package shows the result, with an action to open the novel on success
+AC-10. Every import creates a new novel, even when the same package was imported before</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3275,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Library screen opened from the sidebar, listing all novels with search, filter, and sort. Opening a novel shows its detail page, the entry point for editing, chapters, export, and reading.</t>
+          <t>Library screen opened from the sidebar, listing all novels with search, filter, and sort. Opening a novel shows its detail page (REQ-023).</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -3273,18 +3285,20 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
           <t>AC-1. Library item in the sidebar is enabled (no longer "Coming soon") and opens the library screen
-AC-2. Each novel shows its cover, title, author, chapter count, and tags
+AC-2. Each novel shows its cover (or a placeholder), title, author, chapter count, and tags
 AC-3. User can search novels by title or author
 AC-4. User can filter novels by tag
-AC-5. User can sort novels by title, author, or import date
+AC-5. User can sort novels by title, author, or import date, ascending or descending
 AC-6. Empty library shows an empty state with an "Import package" action
-AC-7. Opening a novel shows its detail page with metadata and chapter list</t>
+AC-7. A search or filter with no match shows a no-results state with a "Clear filters" action
+AC-8. User can select several novels for a bulk action (delete, REQ-017)
+AC-9. Opening a novel shows its detail page (REQ-023)</t>
         </is>
       </c>
     </row>
@@ -3321,15 +3335,16 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can edit title, author, description, and tags from the novel detail page
+          <t>AC-1. User can edit title, author, description, and tags from the novel detail page and save or cancel the changes
 AC-2. User can replace the cover with a JPG/PNG image or remove it
-AC-3. Title is required; invalid values are rejected with a clear message
-AC-4. Changes are shown in the library screen immediately</t>
+AC-3. Title is required; invalid values (e.g. a cover that is too large or not an image) are rejected with a clear message
+AC-4. Leaving the page with unsaved changes asks for confirmation
+AC-5. Changes are shown in the library screen immediately</t>
         </is>
       </c>
     </row>
@@ -3366,16 +3381,17 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can rename a chapter
-AC-2. User can reorder chapters by drag and drop
-AC-3. User can merge two or more consecutive chapters into one
-AC-4. User can split a chapter into two at a chosen paragraph
-AC-5. User can delete one or many chapters after confirmation</t>
+AC-2. User can reorder chapters by drag and drop or with the keyboard
+AC-3. User can merge two or more consecutive chapters into one; the merged chapter keeps the title of the first
+AC-4. User can split a chapter into two at a chosen paragraph, with a preview of the paragraphs
+AC-5. User can delete one or many chapters after confirmation
+AC-6. A failed merge or split leaves the chapters unchanged</t>
         </is>
       </c>
     </row>
@@ -3412,14 +3428,15 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can delete one or many novels after confirmation
-AC-2. All data of the novel is deleted: files, metadata, chapters, and bookmarks
-AC-3. A novel cannot be deleted while a pipeline (e.g. export) is running on it</t>
+          <t>AC-1. User can delete one or many novels after a confirmation that names the novel or the count
+AC-2. All data of the novel is deleted: files, metadata, and chapters
+AC-3. A novel cannot be deleted while a pipeline (e.g. export) is running on it (TSK-024)
+AC-4. Deleting from the detail page returns to the library screen</t>
         </is>
       </c>
     </row>
@@ -3456,53 +3473,90 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can export a novel from its detail page and choose where to save the .zip
+          <t>AC-1. User can export a novel from its detail page and choose where to save the .zip; the default file name is the novel title
 AC-2. Export runs as a pipeline run and appears in the pipeline monitor and history
 AC-3. The exported package follows the format spec (TSK-012) with the current metadata, cover, and chapters in their current order
-AC-4. The exported package keeps the novel's package ID
-AC-5. Importing the exported package into an empty library gives the same metadata and chapters (round trip)</t>
+AC-4. Importing the exported package into an empty library gives the same metadata and chapters (round trip)
+AC-5. A failed or cancelled export leaves no partial .zip file
+AC-6. When the export finishes, a notification offers to show the file in its folder</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="1" t="n"/>
-      <c r="D11" s="1" t="n"/>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>REQ-023</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Novel Detail Page</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Show one novel and give access to all its actions</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Page opened from the library screen (REQ-014). Shows the novel's metadata and chapter list, and is the entry point for reading (REQ-019), editing (REQ-015), chapter management (REQ-016), export (REQ-018), and delete (REQ-017).</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. Page shows cover, title, author, description, tags, language, chapter count, and import date
+AC-2. Page lists all chapters in order; selecting a chapter opens it in the reader
+AC-3. Page has Read, Edit, Export, and Delete actions
+AC-4. Page shows loading, error, and not-found states
+AC-5. Page shows when a pipeline is running on the novel, and actions blocked by it are disabled with the reason (TSK-024)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="105.6" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>REQ-019</t>
+          <t>TSK-024</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>Novel Reader</t>
+          <t>Novel Pipeline Lock</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>Let users read a novel chapter by chapter</t>
+          <t>Keep a novel consistent while a pipeline works on it</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Reader screen opened from the novel detail page, with a table of contents, next/previous navigation, and keyboard shortcuts.</t>
+          <t>Pipeline runs record which novel they work on (TSK-008). While a run on a novel is queued or running, the novel is locked: no metadata edit (REQ-015), chapter change (REQ-016), or delete (REQ-017).</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
@@ -3512,173 +3566,211 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User can open the reader from the novel detail page or from a chapter in the chapter list
-AC-2. Table of contents lists all chapters; selecting a chapter opens it
-AC-3. User can go to the next/previous chapter with buttons and keyboard shortcuts
-AC-4. Each paragraph of the plain-text chapter is shown as a separate paragraph
-AC-5. Reader colors follow the app theme (light/dark)</t>
+          <t>AC-1. Each pipeline run on a novel records the novel's ID
+AC-2. While a run on a novel is queued or running, edit, chapter change, and delete of that novel are refused with a clear reason
+AC-3. The lock is released when the run succeeds, fails, or is cancelled, and after an app restart
+AC-4. Reading and searching a locked novel still work</t>
         </is>
       </c>
     </row>
     <row r="13" ht="79.2" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>TSK-025</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Library File Access for the UI</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Let the UI show covers and chapter text stored in the library</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>The renderer cannot read files directly (AD-06). Main serves library files (covers, chapter text) to the renderer in a safe way, limited to &lt;app data&gt;/library.</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. The UI can show a novel's cover and load a chapter's text
+AC-2. Only files inside &lt;app data&gt;/library can be read; other paths are refused
+AC-3. The page security policy is not weakened to allow other file access</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="79.2" customHeight="1">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="1" t="n"/>
+      <c r="D14" s="1" t="n"/>
+      <c r="E14" s="1" t="n"/>
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="n"/>
+      <c r="H14" s="1" t="n"/>
+    </row>
+    <row r="15" ht="66" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>REQ-019</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Novel Reader</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Let users read a novel chapter by chapter</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Reader screen opened from the novel detail page, with a table of contents, next/previous navigation, and keyboard shortcuts.</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. User can open the reader from the novel detail page or from a chapter in the chapter list
+AC-2. Table of contents lists all chapters and shows the current one; selecting a chapter opens it
+AC-3. User can go to the next/previous chapter with buttons and keyboard shortcuts; they are disabled on the first/last chapter, and shortcuts do not fire while typing in a field
+AC-4. Each paragraph of the plain-text chapter is shown as a separate paragraph
+AC-5. Reader colors follow the app theme (light/dark)
+AC-6. Reader shows the chapter position (e.g. "Chapter 12 / 340")
+AC-7. A chapter whose file is missing shows an error state instead of failing</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
           <t>REQ-020</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Reading Settings</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Let users adjust how chapter text is displayed</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>From the reader, the user changes the font, font size, line height, and content width. Settings apply to all novels and are saved in settings.json.</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
-        <is>
-          <t>1. Draft</t>
-        </is>
-      </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can change font, font size, line height, and content width from the reader
 AC-2. Changes apply immediately to the open chapter
 AC-3. Settings apply to all novels and persist across restarts in settings.json (TSK-010)
-AC-4. User can reset reading settings to default values</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="79.2" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>REQ-021</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
+AC-4. User can reset reading settings to default values
+AC-5. Fonts are bundled with the app (work offline) and support Vietnamese; each numeric setting has a min, max, and step</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>REQ-022</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>Bookmarks</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Let users mark positions in a novel and return to them</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>In the reader, the user bookmarks the current paragraph and opens a novel's bookmark list to jump back.</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Search in Novel</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Let users find text across the chapters of a novel</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>In the reader, the user searches text in all chapters of the open novel and jumps to a result.</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G14" s="1" t="inlineStr">
-        <is>
-          <t>1. Draft</t>
-        </is>
-      </c>
-      <c r="H14" s="1" t="inlineStr">
-        <is>
-          <t>AC-1. User can add a bookmark at a paragraph in the reader
-AC-2. Bookmark list of the novel shows the chapter title and a text snippet; selecting a bookmark opens that position
-AC-3. User can delete bookmarks
-AC-4. Bookmarks stay on the same paragraph after chapters are renamed, reordered, merged, or split; bookmarks of deleted chapters are removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="66" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>REQ-022</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Reader</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>Search in Novel</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Let users find text across the chapters of a novel</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>In the reader, the user searches text in all chapters of the open novel and jumps to a result.</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="G15" s="1" t="inlineStr">
-        <is>
-          <t>1. Draft</t>
-        </is>
-      </c>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can search text across all chapters of the open novel
 AC-2. Search is case-insensitive
-AC-3. Results are grouped by chapter and show a snippet with the match highlighted
-AC-4. Selecting a result opens the chapter at the match</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-      <c r="G16" s="1" t="n"/>
-      <c r="H16" s="1" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n"/>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="1" t="n"/>
-      <c r="D17" s="1" t="n"/>
-      <c r="E17" s="1" t="n"/>
-      <c r="F17" s="1" t="n"/>
-      <c r="G17" s="1" t="n"/>
-      <c r="H17" s="1" t="n"/>
+AC-3. Results are grouped by chapter, show a snippet with the match highlighted, and show the total count
+AC-4. Selecting a result opens the chapter at the match and keeps it highlighted
+AC-5. Search shows searching and no-results states; a new query cancels the previous one</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -3870,10 +3962,30 @@
       <c r="G36" s="1" t="n"/>
       <c r="H36" s="1" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="n"/>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="1" t="n"/>
+      <c r="C38" s="1" t="n"/>
+      <c r="D38" s="1" t="n"/>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REQ014): Browse and inspect library novels
- feat(library): list novels from metadata files and serve covers to the UI [REQ-014]
- feat(library): library screen with filters, grid and list views, and an inspector [REQ-014]
- fix(library): resolve review and test findings [REQ-014]
- docs(library): document the library screen [REQ-014]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2892" yWindow="8220" windowWidth="27648" windowHeight="14952" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1536" yWindow="1536" windowWidth="34560" windowHeight="18684" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity Catalog" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TH-03 Library Management'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Decisions'!$A$1:$J$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -115,7 +115,74 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -800,7 +867,7 @@
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
@@ -3291,7 +3358,7 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -3496,7 +3563,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="92.40000000000001" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
           <t>TSK-025</t>
@@ -3692,7 +3759,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="145.2" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>REQ-023</t>
@@ -3740,7 +3807,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="171.6" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>REQ-016</t>
@@ -3789,7 +3856,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="132" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
           <t>REQ-026</t>
@@ -4065,21 +4132,20 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="6" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="27.6" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Decision ID</t>
@@ -4131,7 +4197,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="26.4" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>AD-01</t>
@@ -4183,7 +4249,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="26.4" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>AD-02</t>
@@ -4235,7 +4301,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="92.40000000000001" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>AD-03</t>
@@ -4288,7 +4354,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="92.40000000000001" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>AD-04</t>
@@ -4342,7 +4408,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="79.2" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>AD-05</t>
@@ -4396,7 +4462,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="66" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>AD-06</t>
@@ -4449,7 +4515,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="66" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
           <t>AD-07</t>
@@ -4504,7 +4570,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="79.2" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>AD-08</t>
@@ -4559,7 +4625,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="66" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>AD-09</t>
@@ -4614,7 +4680,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="79.2" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
           <t>AD-10</t>
@@ -4668,7 +4734,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="92.40000000000001" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>AD-11</t>
@@ -4722,7 +4788,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="92.40000000000001" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>AD-12</t>
@@ -4775,7 +4841,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="79.2" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>AD-13</t>
@@ -4861,7 +4927,7 @@
       <c r="I15" s="1" t="n"/>
       <c r="J15" s="1" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="26.4" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>AD-15</t>
@@ -4957,7 +5023,7 @@
       <c r="I18" s="1" t="n"/>
       <c r="J18" s="1" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="52.8" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
           <t>AD-18</t>
@@ -5010,7 +5076,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="52.8" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
           <t>AD-19</t>
@@ -5064,7 +5130,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="52.8" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
           <t>AD-20</t>
@@ -5118,7 +5184,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="52.8" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
           <t>AD-21</t>
@@ -5171,7 +5237,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="66" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
           <t>AD-22</t>
@@ -5224,7 +5290,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="79.2" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>AD-23</t>
@@ -5277,7 +5343,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="79.2" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
           <t>AD-24</t>
@@ -5330,7 +5396,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="39.6" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
           <t>AD-25</t>
@@ -5383,7 +5449,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="66" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
           <t>AD-26</t>
@@ -5436,7 +5502,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="66" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
           <t>AD-27</t>
@@ -5489,7 +5555,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="66" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
           <t>AD-28</t>
@@ -5542,7 +5608,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="79.2" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>AD-29</t>
@@ -5595,7 +5661,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="52.8" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
         <is>
           <t>AD-30</t>
@@ -5648,7 +5714,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="39.6" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
           <t>AD-31</t>
@@ -5701,7 +5767,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="52.8" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
           <t>AD-32</t>
@@ -5754,7 +5820,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="52.8" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
         <is>
           <t>AD-33</t>
@@ -5807,7 +5873,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="79.2" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
         <is>
           <t>AD-34</t>
@@ -5860,7 +5926,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="66" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
           <t>AD-35</t>
@@ -5913,7 +5979,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="52.8" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
           <t>AD-36</t>
@@ -5966,7 +6032,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="66" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
           <t>AD-37</t>
@@ -6019,7 +6085,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="52.8" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
           <t>AD-38</t>

</xml_diff>

<commit_message>
feat(REQ018): Export a novel to a Dreamer package from the library inspector as a background pipeline, and read chapter text over IPC (TSK-025)
- Drop TSK-024 from TH03-02 (lock rules kept in REQ-017, REQ-023, REQ-026)
- library:get-chapter returns the paragraphs of a chapter listed in the novel (TSK-025); library:get returns the chapter list
- Pipeline novel-export: native Save dialog, <target>.zip.tmp + rename, cleanup on fail / cancel / app close, novel locked while it runs
- Inspector Export with Exporting / Exported (Show in folder) / Couldn't export toasts
- Overview and CLAUDE.md updated; REQ-018, TSK-025, TH03-02 set to Done

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -908,7 +908,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -3105,7 +3105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>The user deletes the active novel from the inspector of the library screen (REQ-014), or many novels with multi-select. A bulk delete skips locked novels (TSK-024).</t>
+          <t>The user deletes the active novel from the inspector of the library screen (REQ-014), or many novels with multi-select. A bulk delete skips novels a pipeline is running on.</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
         <is>
           <t>AC-1. User can delete one or many novels after a confirmation that names the novel, or says how many novels will be deleted
 AC-2. All data of the novel is deleted: files, metadata, and chapters
-AC-3. A novel cannot be deleted while a pipeline (e.g. export) is running on it (TSK-024); a bulk delete skips locked novels and the confirmation names the skipped ones</t>
+AC-3. A novel cannot be deleted while a pipeline (e.g. export) is running on it; a bulk delete skips locked novels and the confirmation names the skipped ones</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3504,7 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -3521,7 +3521,7 @@
     <row r="10" ht="118.8" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>TSK-024</t>
+          <t>TSK-025</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -3531,17 +3531,17 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Novel Pipeline Lock</t>
+          <t>Library File Access for the UI</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Keep a novel consistent while a pipeline works on it</t>
+          <t>Let the UI show covers and chapter text stored in the library</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Pipeline runs record which novel they work on (TSK-008). While a run on a novel is queued or running, the novel is locked: no metadata edit (REQ-015), chapter change (REQ-016), chapter edit (REQ-026), or delete (REQ-017).</t>
+          <t>The renderer cannot read files directly (AD-06). Main serves library files (covers, chapter text) to the renderer in a safe way, limited to &lt;app data&gt;/library, and a preview of a cover image the user just picked, before save.</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
@@ -3551,55 +3551,10 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>AC-1. Each pipeline run on a novel records the novel's ID
-AC-2. While a run on a novel is queued or running, edit, chapter change, chapter edit, and delete of that novel are refused with a clear reason
-AC-3. The lock is released when the run succeeds, fails, or is cancelled, and after an app restart
-AC-4. Reading and searching a locked novel still work</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="92.40000000000001" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>TSK-025</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>Library File Access for the UI</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Let the UI show covers and chapter text stored in the library</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>The renderer cannot read files directly (AD-06). Main serves library files (covers, chapter text) to the renderer in a safe way, limited to &lt;app data&gt;/library, and a preview of a cover image the user just picked, before save.</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="inlineStr">
-        <is>
-          <t>2. Approve</t>
-        </is>
-      </c>
-      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>AC-1. The UI can show a novel's cover, a preview of a cover image the user just picked (before save), and load a chapter's text, without the renderer reading files outside &lt;app data&gt;/library
 AC-2. Only files inside &lt;app data&gt;/library can be read; other paths are refused
@@ -3607,53 +3562,53 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="92.40000000000001" customHeight="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+    </row>
     <row r="12" ht="105.6" customHeight="1">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="1" t="n"/>
-      <c r="D12" s="1" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-      <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
-    </row>
-    <row r="13" ht="79.2" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>REQ-019</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Novel Reader</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>Let users read a novel chapter by chapter</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Reader in the center of the novel detail page (REQ-023); the Chapters panel is the table of contents. Next/previous navigation, keyboard shortcuts, and a Focus mode.</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H12" s="1" t="inlineStr">
         <is>
           <t>AC-1. Opening a novel shows its first chapter in the reader (no auto resume in 0.1.0)
 AC-2. The Chapters panel is the table of contents: it lists all chapters and marks the current one; selecting a chapter opens it
@@ -3666,43 +3621,43 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="79.2" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="13" ht="79.2" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>REQ-020</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Reading Settings</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>Let users adjust how chapter text is displayed</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>In the Reading tab of the novel detail page (REQ-023), the user changes the font, font size, line height, and content width. Settings apply to all novels and are saved in settings.json.</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G14" s="1" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can change font, font size, line height, and content width in the Reading tab
 AC-2. Changes apply immediately to the open chapter
@@ -3712,43 +3667,43 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="66" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="14" ht="79.2" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>REQ-022</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Search in Novel</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>Let users find text across the chapters of a novel</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>In the Search tab of the novel detail page (REQ-023), the user searches text in all chapters of the novel and jumps to a result.</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G15" s="1" t="inlineStr">
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can search text across all chapters of the open novel
 AC-2. Search is case-insensitive
@@ -3759,43 +3714,43 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="145.2" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="15" ht="66" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>REQ-023</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Novel Detail Page</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>Show one novel as a reader with its chapters</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Page opened from the library screen (REQ-014), with a reader layout: Chapters panel on the left (chapter list, search, Organize mode of REQ-016), chapter reader in the center (REQ-019), and a right panel with the Reading (REQ-020) and Search (REQ-022) tabs. Metadata, export, and delete stay in the library screen.</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G16" s="1" t="inlineStr">
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H16" s="1" t="inlineStr">
+      <c r="H15" s="1" t="inlineStr">
         <is>
           <t>AC-1. Top bar breadcrumb shows "Library · Novels · &lt;novel title&gt;"
 AC-2. Page header shows the current chapter (e.g. "0012 · &lt;chapter title&gt;") and only two actions: Edit (REQ-026) and Focus (REQ-019)
@@ -3803,47 +3758,47 @@
 AC-4. Chapters panel search: digits search by chapter number and Enter opens that chapter; text filters the list by chapter title
 AC-5. Right panel has the Reading (REQ-020) and Search (REQ-022) tabs
 AC-6. Page shows loading, error, and not-found states
-AC-7. Page shows a banner when a pipeline is running on the novel; Edit is disabled with the reason (TSK-024)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="171.6" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
+AC-7. Page shows a banner when a pipeline is running on the novel; Edit is disabled with the reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="145.2" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>REQ-016</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Chapter Management</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Let users organize the chapters of a novel</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>In the Organize mode of the Chapters panel on the novel detail page (REQ-023), the user renames, reorders, merges, splits, and deletes chapters. Each change is saved at once.</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G17" s="1" t="inlineStr">
+      <c r="G16" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="H16" s="1" t="inlineStr">
         <is>
           <t>AC-1. User can rename a chapter
 AC-2. User can reorder chapters by drag and drop or with the keyboard
@@ -3856,43 +3811,43 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="132" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="17" ht="171.6" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>REQ-026</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Edit Chapter</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>Let users fix the title and text of a chapter</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t>Edit in the header of the novel detail page (REQ-023) opens an editor for the current chapter's title and text in place of the reader (REQ-019). Refused while the novel is locked (TSK-024).</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Edit in the header of the novel detail page (REQ-023) opens an editor for the current chapter's title and text in place of the reader (REQ-019). Refused while a pipeline is running on the novel.</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="G18" s="1" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>2. Approve</t>
         </is>
       </c>
-      <c r="H18" s="1" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>AC-1. Edit opens an editor for the current chapter's title and text in place of the reader; the text shows one paragraph per line
 AC-2. Editor has Save and Cancel; Save is disabled until something changes
@@ -3900,9 +3855,19 @@
 AC-4. After save, the reader shows the new title and text, and the chapter's character and paragraph counts are updated
 AC-5. Cancelling or leaving the page with unsaved changes asks for confirmation
 AC-6. The Chapters panel and the Search tab are disabled while editing
-AC-7. Edit is refused while the novel is locked (TSK-024)</t>
-        </is>
-      </c>
+AC-7. Edit is refused while a pipeline is running on the novel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="132" customHeight="1">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="n"/>
+      <c r="C18" s="1" t="n"/>
+      <c r="D18" s="1" t="n"/>
+      <c r="E18" s="1" t="n"/>
+      <c r="F18" s="1" t="n"/>
+      <c r="G18" s="1" t="n"/>
+      <c r="H18" s="1" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -4104,20 +4069,10 @@
       <c r="G38" s="1" t="n"/>
       <c r="H38" s="1" t="n"/>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
-      <c r="G39" s="1" t="n"/>
-      <c r="H39" s="1" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(REQ019): Read a novel chapter by chapter on the novel page, with a chapter list, pager, shortcuts and Focus mode
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -3605,7 +3605,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>3. Implement</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(REQ026): Edit the title and text of the current chapter on the novel page, with an unsaved-changes guard, saved as a new content-hash file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -3747,7 +3747,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>3. Implement</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">

</xml_diff>

<commit_message>
chore(solu): setting page with LLM integrations
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -3,21 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1536" yWindow="1536" windowWidth="34560" windowHeight="18684" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5760" yWindow="5760" windowWidth="34560" windowHeight="18684" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity Catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-01 Foundation" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-02 Configuration" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-03 Library Management" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-04 Library Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Capacity Catalog'!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TH-01 Foundation'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TH-02 Configuration'!$A$1:$H$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TH-03 Library Management'!$A$1:$H$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Open Decisions'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TH-04 Library Analysis'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Open Decisions'!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -776,106 +778,70 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>TH-02 Configuration - LLM Integrations - LLM Provider Setup</t>
+          <t>TH-02 Configuration - LLM Integrations - LLM Integrations</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Detect and configure LLM providers</t>
+          <t>Set up the LLM providers and choose the LLM used by each feature</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>cross-release</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>0. Idea</t>
+          <t>1. Draft</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>Detects LLM CLIs installed on the machine (Codex, Claude, Antigravity) and lets the user add cloud providers (OpenAI, Anthropic, Google) with an API key. Prerequisite for the Analysis features in 0.2.0.</t>
+          <t>Detects LLM CLIs installed on the machine, lets the user add cloud LLM providers, and tests each one. The user picks one default LLM (provider and model) and, optionally, another LLM per feature. Requirements are added in the release of the main feature that needs them; each requirement states which providers and features it covers.</t>
         </is>
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>1. check and show installed LLM CLI (Codex, Claude, Antigravity)
-2. add cloud providers for LLM (OpenAI, Anthropic, Google)
-3. test connection per provider</t>
+          <t>1. show the available LLM providers (installed CLIs, cloud providers)
+2. configure and test each provider
+3. one default LLM, and an LLM per feature that uses one; a feature without its own choice uses the default
+4. requirements added with the main features that need them</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26.4" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>TH02-04</t>
+          <t>TH03-01</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>TH-02 Configuration - LLM Integrations - LLM Integrations per Feature</t>
+          <t>TH-03 Library Management - Novel Management - Library: Novel Import Package</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Select integration per feature</t>
+          <t>Import novels into the library from a Dreamer package (.zip)</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>cross-release</t>
+          <t>0.1.0</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>0. Idea</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>Lets the user pick a provider/model per feature (World Graph, Translation, etc.). Expanded gradually with each release.</t>
+          <t>Defines the Dreamer package format (.zip with metadata.json, an optional cover, and chapters/*.txt) and imports one package at a time from an Import screen. The package type comes from metadata.json (only novel in 0.1.0). The package is read and checked without writing anything, the user reviews and edits a preview, then the import runs as a background pipeline. Every import creates a new novel; there is no duplicate check and no import into an existing novel. Each novel is stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/: metadata.json (metadata and chapter list), cover, and chapter text; nothing of the library is stored in SQLite (TSK-013, AD-38). The same format is used by Export (TH03-02).</t>
         </is>
       </c>
       <c r="G9" s="1" t="inlineStr">
-        <is>
-          <t>1. select LLM integration per feature</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="92.40000000000001" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>TH03-01</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>TH-03 Library Management - Novel Management - Library: Novel Import Package</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>Import novels into the library from a Dreamer package (.zip)</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>4. Done</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>Defines the Dreamer package format (.zip with metadata.json, an optional cover, and chapters/*.txt) and imports one package at a time from an Import screen. The package type comes from metadata.json (only novel in 0.1.0). The package is read and checked without writing anything, the user reviews and edits a preview, then the import runs as a background pipeline. Every import creates a new novel; there is no duplicate check and no import into an existing novel. Each novel is stored as files in &lt;app data&gt;/library/&lt;novel-uuid&gt;/: metadata.json (metadata and chapter list), cover, and chapter text; nothing of the library is stored in SQLite (TSK-013, AD-38). The same format is used by Export (TH03-02).</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>1. Dreamer package format (.zip) defined, versioned, and documented in _docs
 2. Import screen opened from Home and Library: pick or drop one package, check it, preview and edit, then import as a background pipeline
@@ -885,38 +851,38 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="66" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="10" ht="92.40000000000001" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>TH03-02</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Operations</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Browse and manage the novels in the library</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>4. Done</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>Library screen listing all imported novels in a grid or list, with a Filters panel (search, sort, language, publication status, genre) and an inspector for the active novel. From the inspector the user edits a novel's metadata (title, author, cover, tags, description, publication status), deletes novels, exports a novel to a Dreamer package, opens its folder, and opens its detail page (TH03-03). Analysed / Translated counts and filters and the Musics / Videos tabs are shown as "Coming soon" (TH04 or later).</t>
         </is>
       </c>
-      <c r="G11" s="1" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>1. library screen lists novels in a grid or list with search, filters (language, publication status, genre), and sort
 2. inspector for the active novel with its stats, metadata, and actions
@@ -926,38 +892,38 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="66" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>TH03-03</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>TH-03 Library Management - Novel Management - Library: Novel Detail and Reader</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Read and organize a novel's chapters inside the app</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>2. Approve</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>4. Done</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>Novel detail page opened from the library screen, built as a reader: Chapters panel on the left (table of contents, search, Organize mode), chapter reader in the center, and Reading / Search tabs on the right. The user reads chapter by chapter with next/previous navigation, keyboard shortcuts, and a Focus mode; manages chapters (rename, reorder, merge, split, delete); edits the current chapter's title and text; changes reading settings (font, font size, line height, content width) that apply to all novels; and searches text across the novel's chapters. No bookmarks and no auto resume in 0.1.0.</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>1. novel detail page with Chapters panel, reader, and Reading / Search tabs
 2. chapter navigation (next/previous, keyboard shortcuts) and Focus mode
@@ -968,18 +934,65 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>TH04-01</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Build an accurate, editable world of a novel from its chapters</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>The Analysis page (sidebar, Analysis group) runs World Analysis on a novel and shows its world. The pipeline analyses chapters one by one: Preparation (code) → Candidates (LLM: entities named with exact words from the text: characters, personas, locations, organizations, glossary terms) → Predicates (LLM: facts about entities, a relationship or a scalar value, each backed by an exact quote) → Verification (code: words and quotes exist in the chapter, types and values follow ontology.yml) → Review (human, optional). Results are saved per chapter; verified results merge into the novel's world automatically. The page shows the pipeline progress and results, and the Novel World as a graph of one analysed chapter or of the whole novel (Omniscient mode). The user edits the world freely; user edits always win over re-runs. ontology.yml has an app default, copied per novel and edited as a file. The novel is locked while the pipeline runs.</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>1. Analysis page in the sidebar with a novel selector
+2. ontology.yml with an app default and a per-novel copy the user edits
+3. run analysis from a dialog: missing chapters, chapter range, or full; overwrite option for range and full
+4. pipeline progress and per-chapter results with exact words and quotes, verified by code
+5. verified results merge into the world automatically; optional review and fix per chapter
+6. Novel World graph of one analysed chapter, or of the whole novel (Omniscient mode)
+7. user edits the world freely; edits survive re-runs</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="39.6" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>TH04-01</t>
+          <t>TH04-05</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="n"/>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Translate a novel's glossary and chapters with an LLM, consistently</t>
+        </is>
+      </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
           <t>0.2.0</t>
@@ -987,83 +1000,84 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
+          <t>2. Approve</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>Use an LLM to analyze a section of a novel and produce an omniscient world graph: characters, personas, locations, organizations, and glossary.</t>
-        </is>
-      </c>
-      <c r="G13" s="1" t="n"/>
+          <t>Glossary of all entity names and aliases from the novel's world (TH04-01), translated by an LLM into a target language (English or Vietnamese, not the source language); the user edits any translation. A pipeline then translates the chapters, started from a dialog like World Analysis (missing chapters, chapter range, or full, with an overwrite option). Each chapter is translated with the glossary entries found in it, and code checks the result against the glossary (dictionary check). Glossary and chapter translation share one instruction the user defines per novel and target language. Several target languages are kept side by side. The reader shows the original, the translation, or both; the user edits a translation and the check runs again. The novel is locked while a pipeline runs.</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>1. one translation instruction per novel and target language, shared by glossary and chapter translation
+2. glossary of the world's names with one translation per target language; LLM translation as a pipeline; user translations kept on re-runs
+3. run chapter translation from a dialog: target language, missing chapters, chapter range, or full; overwrite option
+4. each chapter translated with the glossary entries found in it; deterministic dictionary check after
+5. reader shows the original, the translation, or side by side; user edits a translation
+6. translation status per chapter, language, and novel</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26.4" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>TH04-04</t>
+          <t>TH03-04</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Glossary Translation</t>
+          <t>TH-03 Library Management - Music Management - Library: Music Operations</t>
         </is>
       </c>
       <c r="C14" s="1" t="n"/>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>Based on the entities identified in the novel world graph, provide translated versions of those entities.</t>
-        </is>
-      </c>
+          <t>0. Idea</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n"/>
       <c r="G14" s="1" t="n"/>
     </row>
     <row r="15" ht="39.6" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>TH04-05</t>
+          <t>TH03-05</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Content Translation</t>
+          <t>TH-03 Library Management - Music Management - Library: Music Viewer</t>
         </is>
       </c>
       <c r="C15" s="1" t="n"/>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>0.2.0</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>1. Draft</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>Use an LLM to translate each chapter of the novel, based on the entities appearing in that chapter and their glossary translations.</t>
-        </is>
-      </c>
+          <t>0. Idea</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="n"/>
       <c r="G15" s="1" t="n"/>
     </row>
     <row r="16" ht="26.4" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>TH03-04</t>
+          <t>TH03-06</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Music Management - Library: Music Operations</t>
+          <t>TH-03 Library Management - Video Management - Library: Video Import Package</t>
         </is>
       </c>
       <c r="C16" s="1" t="n"/>
@@ -1083,12 +1097,12 @@
     <row r="17" ht="26.4" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>TH03-05</t>
+          <t>TH03-07</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Music Management - Library: Music Viewer</t>
+          <t>TH-03 Library Management - Video Management - Library: Video Operations</t>
         </is>
       </c>
       <c r="C17" s="1" t="n"/>
@@ -1108,12 +1122,12 @@
     <row r="18" ht="26.4" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>TH03-06</t>
+          <t>TH03-08</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Video Management - Library: Video Import Package</t>
+          <t>TH-03 Library Management - Video Management - Library: Video Viewer</t>
         </is>
       </c>
       <c r="C18" s="1" t="n"/>
@@ -1133,12 +1147,12 @@
     <row r="19" ht="26.4" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>TH03-07</t>
+          <t>TH04-02</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Video Management - Library: Video Operations</t>
+          <t xml:space="preserve">TH-04 Library Analysis - Music Insight Analysis - </t>
         </is>
       </c>
       <c r="C19" s="1" t="n"/>
@@ -1158,12 +1172,12 @@
     <row r="20" ht="26.4" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>TH03-08</t>
+          <t>TH04-03</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TH-03 Library Management - Video Management - Library: Video Viewer</t>
+          <t xml:space="preserve">TH-04 Library Analysis - Video Insight Analysis - </t>
         </is>
       </c>
       <c r="C20" s="1" t="n"/>
@@ -1183,12 +1197,12 @@
     <row r="21" ht="26.4" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>TH04-02</t>
+          <t>TH05-01</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-04 Library Analysis - Music Insight Analysis - </t>
+          <t xml:space="preserve">TH-05 Production Projects - Project Management - </t>
         </is>
       </c>
       <c r="C21" s="1" t="n"/>
@@ -1208,12 +1222,12 @@
     <row r="22" ht="26.4" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>TH04-03</t>
+          <t>TH05-02</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-04 Library Analysis - Video Insight Analysis - </t>
+          <t xml:space="preserve">TH-05 Production Projects - Scripting - </t>
         </is>
       </c>
       <c r="C22" s="1" t="n"/>
@@ -1233,12 +1247,12 @@
     <row r="23" ht="26.4" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>TH05-01</t>
+          <t>TH05-03</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Production Projects - Project Management - </t>
+          <t xml:space="preserve">TH-05 Production Projects - Worldbuilding - </t>
         </is>
       </c>
       <c r="C23" s="1" t="n"/>
@@ -1258,12 +1272,12 @@
     <row r="24" ht="26.4" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>TH05-02</t>
+          <t>TH05-04</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Production Projects - Scripting - </t>
+          <t xml:space="preserve">TH-05 Production Projects - Storyboards - </t>
         </is>
       </c>
       <c r="C24" s="1" t="n"/>
@@ -1283,12 +1297,12 @@
     <row r="25" ht="26.4" customHeight="1">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>TH05-03</t>
+          <t>TH05-05</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Production Projects - Worldbuilding - </t>
+          <t xml:space="preserve">TH-05 Production Projects - Canvas - </t>
         </is>
       </c>
       <c r="C25" s="1" t="n"/>
@@ -1308,12 +1322,12 @@
     <row r="26" ht="26.4" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>TH05-04</t>
+          <t>TH05-06</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Production Projects - Storyboards - </t>
+          <t xml:space="preserve">TH-05 Production Projects - Editor - </t>
         </is>
       </c>
       <c r="C26" s="1" t="n"/>
@@ -1333,12 +1347,12 @@
     <row r="27" ht="26.4" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>TH05-05</t>
+          <t>TH06-01</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Production Projects - Canvas - </t>
+          <t xml:space="preserve">TH-06 Media Resources - Sound Effects - </t>
         </is>
       </c>
       <c r="C27" s="1" t="n"/>
@@ -1358,12 +1372,12 @@
     <row r="28" ht="26.4" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>TH05-06</t>
+          <t>TH06-02</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-05 Production Projects - Editor - </t>
+          <t xml:space="preserve">TH-06 Media Resources - Visual Effects - </t>
         </is>
       </c>
       <c r="C28" s="1" t="n"/>
@@ -1383,12 +1397,12 @@
     <row r="29" ht="26.4" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>TH06-01</t>
+          <t>TH07-01</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-06 Media Resources - Sound Effects - </t>
+          <t xml:space="preserve">TH-07 Miscellanouse - Assistant - </t>
         </is>
       </c>
       <c r="C29" s="1" t="n"/>
@@ -1408,12 +1422,12 @@
     <row r="30" ht="26.4" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>TH06-02</t>
+          <t>TH07-02</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TH-06 Media Resources - Visual Effects - </t>
+          <t xml:space="preserve">TH-07 Miscellanouse - Distributions - </t>
         </is>
       </c>
       <c r="C30" s="1" t="n"/>
@@ -1430,56 +1444,8 @@
       <c r="F30" s="1" t="n"/>
       <c r="G30" s="1" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>TH07-01</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TH-07 Miscellanouse - Assistant - </t>
-        </is>
-      </c>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E31" s="1" t="inlineStr">
-        <is>
-          <t>0. Idea</t>
-        </is>
-      </c>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
-    </row>
-    <row r="32" ht="26.4" customHeight="1">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>TH07-02</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TH-07 Miscellanouse - Distributions - </t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="n"/>
-      <c r="D32" s="1" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E32" s="1" t="inlineStr">
-        <is>
-          <t>0. Idea</t>
-        </is>
-      </c>
-      <c r="F32" s="1" t="n"/>
-      <c r="G32" s="1" t="n"/>
-    </row>
+    <row r="31" ht="26.4" customHeight="1"/>
+    <row r="32" ht="26.4" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:G32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2398,7 +2364,7 @@
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
+      <formula1>'Capacity Catalog'!$B$2:$B$30</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2412,7 +2378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2848,27 +2814,100 @@
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="1" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="1" t="n"/>
-      <c r="D12" s="1" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-      <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
+    <row r="12" ht="132" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>REQ-027</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>TH-02 Configuration - LLM Integrations - LLM Integrations</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>LLM CLI Setup</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Let users see and test the LLM CLIs installed on the machine</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>New LLM section in the Settings screen (REQ-006) lists the supported CLIs (Claude Code, Codex, Antigravity), whether each is installed, and its version, with a test per CLI. Cloud providers with an API key are "Coming soon".</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. Settings has an LLM section listing Claude Code, Codex, and Antigravity, each shown as installed (with version) or not installed
+AC-2. Detection runs when the section opens and on demand ("Detect again")
+AC-3. User can set the path of a CLI that is not found automatically; an invalid path is refused with a clear message
+AC-4. "Test" on an installed CLI sends a short prompt and shows OK, or the error with a suggested fix (e.g. not signed in)
+AC-5. Cloud providers (OpenAI, Anthropic, Google) are shown as "Coming soon"
+AC-6. Self-check (TSK-011) adds an LLM check: Warning when no LLM CLI is installed</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="n"/>
-      <c r="G13" s="1" t="n"/>
-      <c r="H13" s="1" t="n"/>
-    </row>
-    <row r="14">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>REQ-028</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>TH-02 Configuration - LLM Integrations - LLM Integrations</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>LLM per Feature</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Let users choose which LLM each analysis feature uses</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>In the LLM section of Settings (REQ-027), the user picks a default LLM (CLI and model) and, optionally, a different one for World Analysis, Glossary Translation, and Content Translation.</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. User picks a default LLM: an installed CLI and a model
+AC-2. User can pick a different LLM for World Analysis, Glossary Translation, and Content Translation; "Use default" is the initial value
+AC-3. Choices are saved in settings.json (TSK-010) and persist across restarts
+AC-4. Each run dialog (REQ-031, REQ-038, REQ-039) shows the LLM it will use
+AC-5. When the chosen LLM is not available, the run is disabled with the reason and a link to the LLM settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="92.40000000000001" customHeight="1">
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="1" t="n"/>
       <c r="C14" s="1" t="n"/>
@@ -3088,11 +3127,31 @@
       <c r="G35" s="1" t="n"/>
       <c r="H35" s="1" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="n"/>
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+      <c r="H36" s="1" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="n"/>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
+    <dataValidation sqref="B2:B37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Capacity Catalog'!$B$2:$B$30</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4073,7 +4132,7 @@
   <autoFilter ref="A1:H36"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Capacity Catalog'!$B$2:$B$32</formula1>
+      <formula1>'Capacity Catalog'!$B$2:$B$30</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4081,6 +4140,708 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="33.5546875" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="20.109375" customWidth="1" min="4" max="4"/>
+    <col width="33.77734375" customWidth="1" min="5" max="5"/>
+    <col width="13.6640625" customWidth="1" min="6" max="6"/>
+    <col width="13.44140625" customWidth="1" min="7" max="7"/>
+    <col width="69.33203125" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Req ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Capacity Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Req Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="158.4" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>REQ-029</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Analysis Page</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Give World Analysis its own page</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>The Analysis item of the sidebar (Analysis group, "Coming soon" until 0.2.0) opens the Analysis page for one novel: a novel selector, the Pipeline area with the analysis progress and results (REQ-032), and the Novel World (REQ-034).</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. The Analysis item in the sidebar is enabled and opens the Analysis page
+AC-2. The page has a novel selector listing the library novels; the last selected novel is kept when the user comes back
+AC-3. "Analyse" in the novel detail page header (REQ-023) and in the library inspector (REQ-014) opens the Analysis page with that novel selected
+AC-4. The page has two areas: Pipeline (progress and results, REQ-032) and Novel World (REQ-034)
+AC-5. Empty states: empty library (with "Import package"), no novel selected, and novel not analysed yet (with "Run analysis")
+AC-6. When no LLM is available, a notice shows the reason with a link to the LLM settings (REQ-027)
+AC-7. Deleting a novel also deletes its analysis data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="171.6" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>REQ-030</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Novel Ontology</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Let users control what World Analysis extracts</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>ontology.yml defines the entity types (character, persona, location, organization, glossary term), the predicate types (a relationship between two entities, or a scalar value of one entity), and their valid values. A default ships with the app and is copied to the novel on its first analysis; the user edits the novel's copy as a file. The format is documented in _docs.</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. The ontology.yml format is documented in _docs: entity types, predicate types with subject and object types, kind (relationship or scalar), and allowed values
+AC-2. The app ships a default ontology covering characters, personas, locations, organizations, and glossary terms
+AC-3. On a novel's first analysis the default is copied to the novel; later analyses of that novel use its copy
+AC-4. From the Analysis page the user opens the novel's ontology.yml in the system editor, and can reset it to the default after a confirmation
+AC-5. An invalid ontology.yml blocks the analysis; the page lists the problems (line and reason)
+AC-6. Changing the ontology does not change existing results; it applies from the next analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="211.2" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>REQ-031</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Run World Analysis</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Let users start World Analysis on a novel</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>"Run analysis" on the Analysis page (REQ-029) opens a dialog to choose the chapters, then starts the World Analysis pipeline: Preparation (code) → Candidates (LLM) → Predicates (LLM) → Verification (code), chapter by chapter.</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. "Run analysis" on the Analysis page opens the run dialog
+AC-2. Dialog options: missing chapters (not analysed, stale, or failed), chapter range (from–to), or full novel
+AC-3. Range and full have an "Overwrite results" checkbox; unchecked, chapters with an up-to-date result are skipped; user edits are never overwritten (REQ-035)
+AC-4. Dialog shows the number of chapters to analyse and the LLM to use (REQ-028); Start is disabled with the reason when there is nothing to run, no LLM is available, or the ontology is invalid
+AC-5. The run appears in the pipeline monitor and history (REQ-004, REQ-005); its log shows the LLM, duration, and token usage when the CLI reports it
+AC-6. While the run is active the novel is locked like for other pipelines (REQ-023 AC-7): chapter, world, and glossary edits are disabled with the reason
+AC-7. Each chapter is saved when it finishes; cancelling keeps the chapters already analysed; a failed chapter does not stop the others
+AC-8. When the run finishes, a notification shows how many chapters were analysed, failed, or have issues, with an action to open the Analysis page</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="171.6" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>REQ-032</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Analysis Progress and Results</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Let users follow the analysis and see the result of each chapter</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline area of the Analysis page (REQ-029): progress of the running analysis and the analysis status of every chapter. The library screen (REQ-014) shows the novel's analysis count.</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. While a run is active, the Pipeline area shows the current chapter and step, chapters done / total, and the failed count, with Cancel
+AC-2. The chapter list shows each chapter's analysis status (not analysed, analysed, has issues, stale, or failed) with an icon and a label, and its counts of entities, facts, and failed items
+AC-3. User can filter the chapter list by status, and select a chapter to review it (REQ-033)
+AC-4. A chapter edited, merged, or split after analysis shows stale or not analysed until it is analysed again
+AC-5. A failed chapter shows the error; "Retry failed" starts a run on the failed chapters
+AC-6. The library inspector shows "Analysed n / N" chapters instead of "Coming soon"; the library Analysed filter is enabled (fully, partly, or not analysed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="198" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>REQ-033</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Chapter Analysis Review</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Let users check and fix the analysis of a chapter</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Selecting a chapter in the Pipeline area (REQ-032) shows its result: the entities found, with the exact words, and the facts, with the exact quote, each verified or failed. Verified items merge into the world automatically; review is optional.</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. Entities show their type (from the ontology) and the exact words used in the chapter for the name and aliases
+AC-2. Facts show a relationship between two entities or a scalar value of one, with the exact quote from the chapter
+AC-3. Each item is verified or failed (icon and label, not color only); a failed item shows the reason: words or quote not found in the chapter, type or predicate not in the ontology, or value not allowed
+AC-4. Matching with the chapter text ignores only differences in Unicode form, whitespace, and quote/dash style, with the same rule as search (REQ-022)
+AC-5. Selecting an item shows its words or quote highlighted in the chapter text
+AC-6. Verified items are in the world; failed items are not, until the user fixes or accepts them
+AC-7. User can reject an item (it leaves the world), fix it within the ontology (it is verified again), or accept a failed item as is; each is saved as a user edit
+AC-8. User can filter items by type and status</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="171.6" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>REQ-034</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Novel World</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Let users explore the world of a novel as a graph</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Novel World area of the Analysis page (REQ-029). Chapter mode shows all entities and relationships of one analysed chapter; Omniscient mode shows all entities and relationships of the whole novel.</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. A mode switch: Chapter (with a selector of analysed chapters) and Omniscient (whole novel)
+AC-2. The graph shows every entity of the mode as a node and every relationship as a link, with its type
+AC-3. User can zoom and pan, filter by entity type and relationship type, and search an entity to highlight it
+AC-4. Selecting a node opens the entity detail: names and aliases, type, scalar values, relationships, and the chapters where it appears; each fact shows its quote
+AC-5. In Omniscient mode the same entity found in several chapters (same name or alias and type) is one node
+AC-6. An entity list next to the graph (search, filter by type, count) gives keyboard and screen-reader access
+AC-7. Items edited by the user are marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="132" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>REQ-035</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Insight Analysis - Analysis: Novel World Graph</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Edit World</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Let users correct the world to fit their needs</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>In the Novel World (REQ-034), the user adds, edits, merges, splits, and deletes entities and facts. User edits are kept apart from LLM results and always win, also on overwrite re-runs.</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. User can add, rename, or delete an entity, and change its type within the ontology
+AC-2. User can add or remove aliases
+AC-3. User can merge two or more entities into one, and split an entity into two
+AC-4. User can add, edit, or delete facts (relationships and scalar values); values follow the ontology
+AC-5. User edits are kept when chapters are analysed again, also with "Overwrite results"
+AC-6. User can reset an edited item to the LLM result
+AC-7. Delete and merge ask for confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="1" t="n"/>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
+      <c r="H9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="105.6" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>REQ-036</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Translation Instruction</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Let users guide the LLM translation of a novel</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>One instruction per novel and target language (e.g. style, forms of address), used by both glossary translation (REQ-038) and chapter translation (REQ-039).</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. User edits the instruction of the novel and a target language from the Glossary view and from both translation dialogs; it is the same text in all three
+AC-2. A new instruction starts from an app default template; the user can reset it to the default
+AC-3. The instruction is used by every glossary and chapter translation of that novel and language
+AC-4. The instruction is saved with the novel, kept across restarts, and deleted with the novel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="171.6" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>REQ-037</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Glossary View</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Let users see and edit the glossary of a novel</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Glossary view of the novel detail page (REQ-023), opened with a Reader / Glossary view switch: a table of the names and aliases of the novel's world (TH04-01) with their translation in the selected target language.</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. The novel detail page has a view switch: Reader, Glossary
+AC-2. The table shows name, entity type, translation, and status (untranslated, LLM, edited by user)
+AC-3. User selects the target language: English or Vietnamese, except the novel's source language
+AC-4. Each entity name and alias of the world is one row; a name added to the world appears as untranslated
+AC-5. User can search and filter by entity type and status
+AC-6. User can edit a translation inline (saved as a user translation) or clear it (back to untranslated)
+AC-7. A novel without analysis shows an empty state with a link to the Analysis page
+AC-8. Deleting a novel also deletes its glossary and translations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="132" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>REQ-038</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Translate Glossary</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Let users translate the glossary with an LLM</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>"Translate glossary" in the Glossary view (REQ-037) opens a dialog, then runs a background pipeline that translates the names with the novel's instruction (REQ-036).</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. The dialog shows the target language, the instruction (REQ-036), the LLM (REQ-028), and the number of names to translate
+AC-2. Options: untranslated names only (default) or all names; user translations are never replaced
+AC-3. The run appears in the pipeline monitor and history; cancelling keeps the translations already saved
+AC-4. While the run is active the novel is locked like for other pipelines (REQ-023 AC-7)
+AC-5. When the run finishes, a notification shows how many names were translated or failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="330" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>REQ-039</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Run Content Translation</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Let users translate the chapters of a novel with an LLM</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>"Translate" in the header of the novel detail page (REQ-023) opens a dialog like World Analysis (REQ-031), then runs the Content Translation pipeline. Each chapter is translated with the instruction (REQ-036) and the glossary entries found in it, then checked against the glossary by code (dictionary check).</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. "Translate" in the novel detail page header opens the run dialog
+AC-2. Dialog options: target language (English or Vietnamese, except the source language); missing chapters (not translated, stale, or failed), chapter range, or full novel
+AC-3. Range and full have an "Overwrite translations" checkbox; when it would replace translations edited by the user, the dialog says how many
+AC-4. The dialog shows the number of chapters, the LLM (REQ-028), and the instruction (REQ-036), and warns when glossary names in those chapters are not translated yet, with a link to the Glossary view; the user can still start
+AC-5. Each chapter title and text is translated with the instruction and the glossary entries found in it; long chapters are translated in parts so they fit the LLM limit
+AC-6. Dictionary check (code, no LLM) after each chapter: each glossary name found in the source chapter must have its translation in the translated text, and the translation must have one paragraph per source paragraph; each miss is an issue; the check runs again when the translation or the glossary changes
+AC-7. The run appears in the pipeline monitor and history; the novel is locked (REQ-023 AC-7); cancelling keeps the translated chapters; a failed chapter does not stop the others
+AC-8. The Chapters panel shows the translation status of each chapter for a selected language: not translated, translated, has issues, stale (source edited after translation), or failed
+AC-9. The library inspector shows "Translated n / N" per language instead of "Coming soon"; the library Translated filter is enabled
+AC-10. When the run finishes, a notification shows how many chapters were translated, failed, or have issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="118.8" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>REQ-040</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Translated Reader</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Let users read a novel in its translation</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>The Reading tab of the novel detail page (REQ-020) gets a display switch: Original, Translation, or Side by side. Dictionary-check issues are shown with the chapter.</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. The Reading tab has a display switch (Original, Translation, Side by side) and a translation language list with only the languages that have translations
+AC-2. Side by side shows each source paragraph next to its translated paragraph
+AC-3. A chapter not translated in the selected language shows an empty state with a "Translate" action
+AC-4. Dictionary-check issues of the chapter are listed; selecting one highlights the source and translated paragraphs
+AC-5. A stale translation shows a notice
+AC-6. The display choice stays when moving between chapters</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="92.40000000000001" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>REQ-041</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>TH-04 Library Analysis - Novel Translation - Analysis: Novel Translation</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Edit Translation</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Let users fix the translation of a chapter</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>When the reader shows a translation (REQ-040), Edit in the page header edits that translation instead of the original, like Edit Chapter (REQ-026).</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>0.2.0</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>2. Approve</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>AC-1. When the reader shows a translation, Edit opens the translated title and text, one paragraph per line
+AC-2. The editor has Save and Cancel; leaving with unsaved changes asks for confirmation
+AC-3. After save, the dictionary check runs again and its issues are updated
+AC-4. A saved translation is marked as edited by the user
+AC-5. Edit is refused while a pipeline is running on the novel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Capacity Catalog'!$B$2:$B$30</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4890,29 +5651,50 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>LLM access layer in Python</t>
+          <t>LLM access layer</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>Provider SDKs vs CLI subprocess (Codex, Claude, Antigravity).</t>
+          <t>Who runs the LLM CLIs (Claude Code, Codex, Antigravity): detect, version, test, and prompts with a JSON schema. 0.2.0 is CLI only (TH02-03, REQ-027).</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>TH02-03, TH02-04</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-      <c r="G16" s="1" t="n"/>
+          <t>TH02-03, REQ-027, REQ-028, TH04-01, TH04-05</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Python backend — One adapter per CLI in Python; main calls it over HTTP like backend jobs (AD-05, AD-34) · cloud SDKs later in the same place
+Electron main (Node) — Main spawns the CLIs directly · works while the backend is down · no HTTP hop · Cons: AI calls leave Python (AD-05), cloud APIs later in Node</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Python backend</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Electron main (Node)</t>
+        </is>
+      </c>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>Deferred</t>
-        </is>
-      </c>
-      <c r="I16" s="1" t="n"/>
-      <c r="J16" s="1" t="n"/>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Human chose Electron main in /solo-solution TH02-03 (2026-10-25). Model: app-shipped suggestions per CLI + free model id. CLIs run in an empty temp folder with tools off / read-only sandbox; text goes in the prompt.</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">

</xml_diff>

<commit_message>
chore(solu): omnisicent page with analyze pipeline
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -962,18 +962,17 @@
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>The Analysis page (sidebar, Analysis group) runs World Analysis on a novel and shows its world. The pipeline analyses chapters one by one: Preparation (code) → Candidates (LLM: entities named with exact words from the text: characters, personas, locations, organizations, glossary terms) → Predicates (LLM: facts about entities, a relationship or a scalar value, each backed by an exact quote) → Verification (code: words and quotes exist in the chapter, types and values follow ontology.yml) → Review (human, optional). Results are saved per chapter; verified results merge into the novel's world automatically. The page shows the pipeline progress and results, and the Novel World as a graph of one analysed chapter or of the whole novel (Omniscient mode). The user edits the world freely; user edits always win over re-runs. ontology.yml has an app default, copied per novel and edited as a file. The novel is locked while the pipeline runs.</t>
+          <t>The Omniscient page (sidebar, Analysis group) runs World Analysis on the current novel and shows its world. The pipeline: Precondition (code) → Candidates (LLM, batches of chapters: entities named with exact words from the text: characters, personas, locations, organizations, glossary terms) → Predicates (LLM, one chapter at a time: facts about entities, a relationship or a scalar value, each backed by an exact quote) → Reviews (code: words and quotes exist in the chapter, types and values follow ontology.yml, no conflicts; the human resolves the issues) → Merge (human: the world is rebuilt from all clean and reviewed chapters). Results are saved per chapter. The page shows the world as a graph or a table up to a chosen chapter, and the review queue. User edits are kept in a world overlay and always win over re-runs. ontology.yml has an app default, copied per novel and edited as a file. The novel is locked while the pipeline runs.</t>
         </is>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>1. Analysis page in the sidebar with a novel selector
+          <t>1. Omniscient page in the sidebar for the current novel chosen in the app top bar
 2. ontology.yml with an app default and a per-novel copy the user edits
-3. run analysis from a dialog: missing chapters, chapter range, or full; overwrite option for range and full
-4. pipeline progress and per-chapter results with exact words and quotes, verified by code
-5. verified results merge into the world automatically; optional review and fix per chapter
-6. Novel World graph of one analysed chapter, or of the whole novel (Omniscient mode)
-7. user edits the world freely; edits survive re-runs</t>
+3. run analysis from a dialog: missing chapters, chapter range, or all; stage, batch size, and overwrite
+4. code checks every chapter result; only chapters with issues are reviewed; merge when every issue is resolved
+5. Novel World as a graph or a table, as of a chosen chapter, with entity details
+6. user edits the world freely in an overlay; edits survive re-runs and merges</t>
         </is>
       </c>
     </row>
@@ -4213,17 +4212,17 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Analysis Page</t>
+          <t>Omniscient Page</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Give World Analysis its own page</t>
+          <t>Give World Analysis and the novel world one page</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>The Analysis item of the sidebar (Analysis group, "Coming soon" until 0.2.0) opens the Analysis page for one novel: a novel selector, the Pipeline area with the analysis progress and results (REQ-032), and the Novel World (REQ-034).</t>
+          <t>The Omniscient item of the sidebar (Analysis group) opens the Omniscient page for the current novel: the views Graph, Table and Review, the entity list, the entity details, and the chapter timeline.</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
@@ -4238,11 +4237,11 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>AC-1. The Analysis item in the sidebar is enabled and opens the Analysis page
-AC-2. The page has a novel selector listing the library novels; the last selected novel is kept when the user comes back
-AC-3. "Analyse" in the novel detail page header (REQ-023) and in the library inspector (REQ-014) opens the Analysis page with that novel selected
-AC-4. The page has two areas: Pipeline (progress and results, REQ-032) and Novel World (REQ-034)
-AC-5. Empty states: empty library (with "Import package"), no novel selected, and novel not analysed yet (with "Run analysis")
+          <t>AC-1. The Omniscient item in the sidebar (Analysis group) is enabled and opens the Omniscient page
+AC-2. The current novel is chosen in the app top bar (novel chip with search) on novel-scoped pages; opening a novel in the library (Open or double-click) makes it the current novel; the choice is kept when the user comes back
+AC-3. "Analyse" in the novel detail page header (REQ-023) and in the library inspector (REQ-014) makes that novel current and opens the Omniscient page
+AC-4. The page has the views Graph, Table and Review, the entity list (left), the entity details (right) and the chapter timeline (bottom, Graph and Table only)
+AC-5. Empty states: empty library (with "Import package") and novel not analysed yet (with "Run analysis")
 AC-6. When no LLM is available, a notice shows the reason with a link to the LLM settings (REQ-027)
 AC-7. Deleting a novel also deletes its analysis data</t>
         </is>
@@ -4287,9 +4286,9 @@
       <c r="H3" s="1" t="inlineStr">
         <is>
           <t>AC-1. The ontology.yml format is documented in _docs: entity types, predicate types with subject and object types, kind (relationship or scalar), and allowed values
-AC-2. The app ships a default ontology covering characters, personas, locations, organizations, and glossary terms
+AC-2. The app ships a default ontology covering characters, personas, locations, organizations, and glossary terms; a character is an abstract entity linked to its personas only by "persona of" (e.g. character Peter Parker has the personas Peter Parker and Spider-Man); every other fact belongs to a persona, location, organization, or glossary term
 AC-3. On a novel's first analysis the default is copied to the novel; later analyses of that novel use its copy
-AC-4. From the Analysis page the user opens the novel's ontology.yml in the system editor, and can reset it to the default after a confirmation
+AC-4. From the Omniscient page the user opens the novel's ontology.yml in the system editor, checks it again, and can reset it to the default after a confirmation
 AC-5. An invalid ontology.yml blocks the analysis; the page lists the problems (line and reason)
 AC-6. Changing the ontology does not change existing results; it applies from the next analysis</t>
         </is>
@@ -4318,7 +4317,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>"Run analysis" on the Analysis page (REQ-029) opens a dialog to choose the chapters, then starts the World Analysis pipeline: Preparation (code) → Candidates (LLM) → Predicates (LLM) → Verification (code), chapter by chapter.</t>
+          <t>"Run analysis" in the Omniscient page toolbar opens a dialog to choose the chapters and parameters, then starts the pipeline: Precondition (code) → Candidates (LLM, batches of chapters) → Predicates (LLM, one chapter at a time) → Reviews (code, REQ-033).</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -4333,14 +4332,17 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>AC-1. "Run analysis" on the Analysis page opens the run dialog
-AC-2. Dialog options: missing chapters (not analysed, stale, or failed), chapter range (from–to), or full novel
-AC-3. Range and full have an "Overwrite results" checkbox; unchecked, chapters with an up-to-date result are skipped; user edits are never overwritten (REQ-035)
-AC-4. Dialog shows the number of chapters to analyse and the LLM to use (REQ-028); Start is disabled with the reason when there is nothing to run, no LLM is available, or the ontology is invalid
-AC-5. The run appears in the pipeline monitor and history (REQ-004, REQ-005); its log shows the LLM, duration, and token usage when the CLI reports it
-AC-6. While the run is active the novel is locked like for other pipelines (REQ-023 AC-7): chapter, world, and glossary edits are disabled with the reason
-AC-7. Each chapter is saved when it finishes; cancelling keeps the chapters already analysed; a failed chapter does not stop the others
-AC-8. When the run finishes, a notification shows how many chapters were analysed, failed, or have issues, with an action to open the Analysis page</t>
+          <t>AC-1. "Run analysis" in the page toolbar opens the run dialog; while a run is active it is replaced by a run pill with Cancel and a link to Pipelines
+AC-2. Dialog modes: missing chapters (not analysed, stale, or failed), chapter range (from–to), or all chapters
+AC-3. Range and all have an "Overwrite results" checkbox; unchecked, chapters with an up-to-date result are skipped; the world overlay is never overwritten (REQ-035)
+AC-4. Stage selects all entity types or one; batch size (1, 3, 5 or 10, default 5) sets how many chapters go to Candidates together; Predicates run one chapter at a time
+AC-5. The dialog shows the chapters to analyse (count and range), the number of batches and the LLM to use (REQ-028); Start is disabled with the reason when there is nothing to run, no LLM is available, or the ontology is invalid
+AC-6. Precondition checks the parameters, the LLM CLI and the novel content before any LLM call
+AC-7. Code checks each LLM result against the ontology and the rules (entity names are exact words of the content); a failing result is asked again up to 3 times, then the last parsable result is kept and its failing items become review issues; an unparsable result fails the chapter
+AC-8. The run appears in the pipeline monitor and history (REQ-004, REQ-005); its log shows the LLM, duration, and token usage when the CLI reports it
+AC-9. While the run is active the novel is locked like for other pipelines (REQ-023 AC-7): chapter, world, review and glossary edits are disabled with the reason
+AC-10. Each chapter is saved when it finishes; cancelling keeps the chapters already analysed; a failed chapter does not stop the others
+AC-11. When the run finishes, a notification shows how many chapters were analysed, failed, or have issues, with an action to open the Omniscient page</t>
         </is>
       </c>
     </row>
@@ -4357,17 +4359,17 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Analysis Progress and Results</t>
+          <t>Analysis Progress and Status</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Let users follow the analysis and see the result of each chapter</t>
+          <t>Let users follow the analysis and see the state of the chapters</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Pipeline area of the Analysis page (REQ-029): progress of the running analysis and the analysis status of every chapter. The library screen (REQ-014) shows the novel's analysis count.</t>
+          <t>Progress of the running analysis and the analysis state of the novel's chapters, shown in the run pill, the chapter timeline and the Review view of the Omniscient page (REQ-029). The library shows the novel's analysis count.</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -4382,11 +4384,11 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>AC-1. While a run is active, the Pipeline area shows the current chapter and step, chapters done / total, and the failed count, with Cancel
-AC-2. The chapter list shows each chapter's analysis status (not analysed, analysed, has issues, stale, or failed) with an icon and a label, and its counts of entities, facts, and failed items
-AC-3. User can filter the chapter list by status, and select a chapter to review it (REQ-033)
-AC-4. A chapter edited, merged, or split after analysis shows stale or not analysed until it is analysed again
-AC-5. A failed chapter shows the error; "Retry failed" starts a run on the failed chapters
+          <t>AC-1. While a run is active, the run pill shows the current chapter and step, chapters done / total and the failed count, with Cancel
+AC-2. Each chapter has an analysis status: not analysed, clean, has issues, reviewed, stale, or failed; the timeline shows "analysed n / N" with the stale, failed and pending-merge counts
+AC-3. Failed chapters are listed in the Review view with their error; "Retry failed" starts a run on them
+AC-4. A chapter edited, merged, or split after analysis shows stale or not analysed until it is analysed again; stale results stay in the world, marked stale; results of deleted chapters leave the world
+AC-5. Stale is found by the chapter file name (content hash) first, then by the chapter index
 AC-6. The library inspector shows "Analysed n / N" chapters instead of "Coming soon"; the library Analysed filter is enabled (fully, partly, or not analysed)</t>
         </is>
       </c>
@@ -4404,17 +4406,17 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Chapter Analysis Review</t>
+          <t>Analysis Review and Merge</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Let users check and fix the analysis of a chapter</t>
+          <t>Let users resolve the analysis issues and build the world from checked results</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Selecting a chapter in the Pipeline area (REQ-032) shows its result: the entities found, with the exact words, and the facts, with the exact quote, each verified or failed. Verified items merge into the world automatically; review is optional.</t>
+          <t>After Candidates and Predicates, code checks the result of every chapter. Chapters without issues are clean and are not reviewed. Chapters with issues are listed in the Review queue; when every issue is resolved, the user merges and the world (world.json) is rebuilt from the results of all clean and reviewed chapters.</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -4429,14 +4431,14 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Entities show their type (from the ontology) and the exact words used in the chapter for the name and aliases
-AC-2. Facts show a relationship between two entities or a scalar value of one, with the exact quote from the chapter
-AC-3. Each item is verified or failed (icon and label, not color only); a failed item shows the reason: words or quote not found in the chapter, type or predicate not in the ontology, or value not allowed
-AC-4. Matching with the chapter text ignores only differences in Unicode form, whitespace, and quote/dash style, with the same rule as search (REQ-022)
-AC-5. Selecting an item shows its words or quote highlighted in the chapter text
-AC-6. Verified items are in the world; failed items are not, until the user fixes or accepts them
-AC-7. User can reject an item (it leaves the world), fix it within the ontology (it is verified again), or accept a failed item as is; each is saved as a user edit
-AC-8. User can filter items by type and status</t>
+          <t>AC-1. Code checks every chapter result: entity names and words exist in the chapter text, quotes exist, types and predicates are in the ontology, values are allowed, and there are no conflicts (for example one name with two types)
+AC-2. A chapter without issues is clean and is not shown for review
+AC-3. The Review queue lists the issues of the chapters with issues, grouped by chapter, each with its reason and the chapter text around the words or quote highlighted
+AC-4. Matching with the chapter text ignores only differences in case, Unicode form, whitespace, and quote/dash style
+AC-5. For each issue the user can reject the item, fix it within the ontology (it is checked again), or accept it when only the words or quote are not found; the fix is saved in that chapter's result
+AC-6. Merge is enabled only when no chapter has an open issue; it rebuilds the world from the results of all clean and reviewed chapters
+AC-7. Analysing a chapter again replaces its result and its previous review; its new issues must be resolved before the next merge
+AC-8. User can filter issues by status, type, and chapter</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4465,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>Novel World area of the Analysis page (REQ-029). Chapter mode shows all entities and relationships of one analysed chapter; Omniscient mode shows all entities and relationships of the whole novel.</t>
+          <t>The Graph and Table views of the Omniscient page (REQ-029) show the world: the merged results (REQ-033) with the world overlay (REQ-035), as of a chosen chapter.</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -4478,13 +4480,14 @@
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>AC-1. A mode switch: Chapter (with a selector of analysed chapters) and Omniscient (whole novel)
-AC-2. The graph shows every entity of the mode as a node and every relationship as a link, with its type
-AC-3. User can zoom and pan, filter by entity type and relationship type, and search an entity to highlight it
-AC-4. Selecting a node opens the entity detail: names and aliases, type, scalar values, relationships, and the chapters where it appears; each fact shows its quote
-AC-5. In Omniscient mode the same entity found in several chapters (same name or alias and type) is one node
-AC-6. An entity list next to the graph (search, filter by type, count) gives keyboard and screen-reader access
-AC-7. Items edited by the user are marked</t>
+          <t>AC-1. The chapter timeline sets "as of chapter N" (the world up to that chapter; default whole novel) and "only this chapter"
+AC-2. The graph shows every entity of the view as a node (colored by type, sized by number of relationships, hubs near the center) and every relationship as a link; hostile relationships are dashed
+AC-3. User can zoom, pan and fit, filter by entity type and relationship type, and search an entity to highlight it; selecting a node highlights it and its neighbours and dims the rest
+AC-4. Selecting an entity opens its details: Entity (names, aliases, type, scalar values per chapter), Relations (with chapters and quotes) and Occurrences (chapters with the text around the name)
+AC-5. The same entity found in several chapters (same name and type, case-insensitive) is one node; aliases never merge entities automatically
+AC-6. The entity list (search, type filter, count) and the Table view (sortable) give keyboard and screen-reader access
+AC-7. Items edited by the user are marked
+AC-8. The world changes only when the user merges (REQ-033); the page shows when it was last merged</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4514,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>In the Novel World (REQ-034), the user adds, edits, merges, splits, and deletes entities and facts. User edits are kept apart from LLM results and always win, also on overwrite re-runs.</t>
+          <t>In the Novel World (REQ-034), the user adds, renames, retypes, merges, splits, and deletes entities, edits aliases, and adds or edits facts. These edits are saved in a world overlay (world-overlay.json), apart from the merged world (REQ-033), and are applied on top of it, so they survive re-runs and merges.</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
@@ -4529,10 +4532,11 @@
           <t>AC-1. User can add, rename, or delete an entity, and change its type within the ontology
 AC-2. User can add or remove aliases
 AC-3. User can merge two or more entities into one, and split an entity into two
-AC-4. User can add, edit, or delete facts (relationships and scalar values); values follow the ontology
-AC-5. User edits are kept when chapters are analysed again, also with "Overwrite results"
-AC-6. User can reset an edited item to the LLM result
-AC-7. Delete and merge ask for confirmation</t>
+AC-4. User can add, edit, or delete facts (relationships and scalar values); values follow the ontology; the quote is optional, and an entered quote must be found in the novel, which ties the fact to that chapter
+AC-5. Edits are saved in the world overlay and applied on top of the merged world; they are kept when chapters are analysed again and when the world is merged again
+AC-6. User can reset an edited item to the merged result
+AC-7. Delete and merge ask for confirmation
+AC-8. An overlay edit that no longer matches the merged world is listed with a warning instead of being dropped</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(solu): translation pages with translation pipeline
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>Glossary of all entity names and aliases from the novel's world (TH04-01), translated by an LLM into a target language (English or Vietnamese, not the source language); the user edits any translation. A pipeline then translates the chapters, started from a dialog like World Analysis (missing chapters, chapter range, or full, with an overwrite option). Each chapter is translated with the glossary entries found in it, and code checks the result against the glossary (dictionary check). Glossary and chapter translation share one instruction the user defines per novel and target language. Several target languages are kept side by side. The reader shows the original, the translation, or both; the user edits a translation and the check runs again. The novel is locked while a pipeline runs.</t>
+          <t>Glossary of all entity names and aliases from the novel's world (TH04-01), translated by an LLM into a target language (English or Vietnamese, not the source language); the user edits any translation. A pipeline then translates the chapters, started from a dialog like World Analysis (missing chapters, chapter range, or full, with an overwrite option). Each chapter is translated with the glossary entries found in it, and code checks the result against the glossary (dictionary check). Glossary and chapter translation share one instruction the user defines per novel and target language. Several target languages are kept side by side. The reader shows the original, the translation, or both; the user edits a translation and the check runs again. The novel is locked while a pipeline runs. Prerequisite: TH04-01 and TH02-03 implemented first.</t>
         </is>
       </c>
       <c r="G13" s="1" t="inlineStr">
@@ -3816,7 +3816,8 @@
 AC-4. Chapters panel search: digits search by chapter number and Enter opens that chapter; text filters the list by chapter title
 AC-5. Right panel has the Reading (REQ-020) and Search (REQ-022) tabs
 AC-6. Page shows loading, error, and not-found states
-AC-7. Page shows a banner when a pipeline is running on the novel; Edit is disabled with the reason</t>
+AC-7. Page shows a banner when a pipeline is running on the novel; Edit is disabled with the reason
+AC-8. (0.2.0) Page header also has the Reader / Glossary view switch (REQ-037) and Translate (REQ-039), shown as a run pill while a translation run is active</t>
         </is>
       </c>
     </row>
@@ -4588,10 +4589,11 @@
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>AC-1. User edits the instruction of the novel and a target language from the Glossary view and from both translation dialogs; it is the same text in all three
+          <t>AC-1. User edits the instruction of the novel and a target language in the right panel of the Glossary view (Save, Reset to default) and in both translation dialogs; it is the same text in all three
 AC-2. A new instruction starts from an app default template; the user can reset it to the default
 AC-3. The instruction is used by every glossary and chapter translation of that novel and language
-AC-4. The instruction is saved with the novel, kept across restarts, and deleted with the novel</t>
+AC-4. The instruction is saved with the novel, kept across restarts, and deleted with the novel
+AC-5. Instruction edits made in a run dialog are saved when the run starts</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4620,7 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>Glossary view of the novel detail page (REQ-023), opened with a Reader / Glossary view switch: a table of the names and aliases of the novel's world (TH04-01) with their translation in the selected target language.</t>
+          <t>Glossary view of the novel detail page (REQ-023), opened with a Reader / Glossary view switch: a table of the names and aliases of the novel's merged world (TH04-01) with their translation in the selected target language, and the instruction (REQ-036) in the right panel.</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -4635,12 +4637,14 @@
         <is>
           <t>AC-1. The novel detail page has a view switch: Reader, Glossary
 AC-2. The table shows name, entity type, translation, and status (untranslated, LLM, edited by user)
-AC-3. User selects the target language: English or Vietnamese, except the novel's source language
-AC-4. Each entity name and alias of the world is one row; a name added to the world appears as untranslated
+AC-3. User selects the target language: English or Vietnamese, except the novel's source language; it is the page's one translation language, also used by the reader and the Chapters panel (REQ-040 AC-7)
+AC-4. Each entity's name and each of its aliases is one row, for all entity types; the same text in two entities is two rows; a name added to the world appears as untranslated
 AC-5. User can search and filter by entity type and status
 AC-6. User can edit a translation inline (saved as a user translation) or clear it (back to untranslated)
 AC-7. A novel without analysis shows an empty state with a link to the Analysis page
-AC-8. Deleting a novel also deletes its glossary and translations</t>
+AC-8. Deleting a novel also deletes its glossary and translations
+AC-9. When a name or alias is no longer in the world (renamed, merged, deleted, alias removed), its translation is dropped
+AC-10. The right panel shows the instruction of the selected language (REQ-036) with Save and Reset to default</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4687,7 @@
       <c r="H12" s="1" t="inlineStr">
         <is>
           <t>AC-1. The dialog shows the target language, the instruction (REQ-036), the LLM (REQ-028), and the number of names to translate
-AC-2. Options: untranslated names only (default) or all names; user translations are never replaced
+AC-2. Options: untranslated names only (default) or all names; user translations are never replaced; batch size of 50 (default), 100, or 200 names per LLM call; the aliases of one entity are always in the same batch
 AC-3. The run appears in the pipeline monitor and history; cancelling keeps the translations already saved
 AC-4. While the run is active the novel is locked like for other pipelines (REQ-023 AC-7)
 AC-5. When the run finishes, a notification shows how many names were translated or failed</t>
@@ -4729,15 +4733,17 @@
       <c r="H13" s="1" t="inlineStr">
         <is>
           <t>AC-1. "Translate" in the novel detail page header opens the run dialog
-AC-2. Dialog options: target language (English or Vietnamese, except the source language); missing chapters (not translated, stale, or failed), chapter range, or full novel
+AC-2. Dialog options: target language (English or Vietnamese, except the source language); missing chapters (not translated, stale, or failed; "has issues" is not missing), chapter range, or full novel; stale chapters are translated again even when edited by the user
 AC-3. Range and full have an "Overwrite translations" checkbox; when it would replace translations edited by the user, the dialog says how many
 AC-4. The dialog shows the number of chapters, the LLM (REQ-028), and the instruction (REQ-036), and warns when glossary names in those chapters are not translated yet, with a link to the Glossary view; the user can still start
-AC-5. Each chapter title and text is translated with the instruction and the glossary entries found in it; long chapters are translated in parts so they fit the LLM limit
-AC-6. Dictionary check (code, no LLM) after each chapter: each glossary name found in the source chapter must have its translation in the translated text, and the translation must have one paragraph per source paragraph; each miss is an issue; the check runs again when the translation or the glossary changes
+AC-5. Each chapter title and text is translated with the instruction and the glossary entries found in it; long chapters are translated in parts, split only at paragraph borders, so they fit the LLM limit
+AC-6. Dictionary check (code, no LLM) after each chapter: each glossary name found in the source chapter must have its translation in the translated text, and the whole translated chapter must have one paragraph per source paragraph; each miss is an issue; the check runs again when the translation or the glossary changes
 AC-7. The run appears in the pipeline monitor and history; the novel is locked (REQ-023 AC-7); cancelling keeps the translated chapters; a failed chapter does not stop the others
-AC-8. The Chapters panel shows the translation status of each chapter for a selected language: not translated, translated, has issues, stale (source edited after translation), or failed
-AC-9. The library inspector shows "Translated n / N" per language instead of "Coming soon"; the library Translated filter is enabled
-AC-10. When the run finishes, a notification shows how many chapters were translated, failed, or have issues</t>
+AC-8. The Chapters panel shows the translation status of each chapter in the page's translation language: not translated, translated, has issues, stale (source chapter changed, or the glossary translation of a name found in it changed), or failed; a changed instruction does not make a chapter stale
+AC-9. The library inspector shows "Translated n / N" for each language that has translations (n = translated + has issues) instead of "Coming soon"; the library Translated filter is enabled, with "Fully translated" and "Partly translated" rows per language, each with a count
+AC-10. When the run finishes, a notification shows how many chapters were translated, failed, or have issues
+AC-11. Glossary names are found with the shared name matcher of TH04-01: case, Unicode form, and quotes are ignored; diacritics are not
+AC-12. A glossary name found in the source with no translation is its own issue, "untranslated name"; the chapter title is checked for names only</t>
         </is>
       </c>
     </row>
@@ -4764,7 +4770,7 @@
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>The Reading tab of the novel detail page (REQ-020) gets a display switch: Original, Translation, or Side by side. Dictionary-check issues are shown with the chapter.</t>
+          <t>A reader bar above the chapter text of the novel detail page (REQ-023) has a display switch: Original, Translation, or Side by side. Dictionary-check issues are listed in a Translation tab of the right panel.</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
@@ -4779,12 +4785,13 @@
       </c>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>AC-1. The Reading tab has a display switch (Original, Translation, Side by side) and a translation language list with only the languages that have translations
+          <t>AC-1. A reader bar above the chapter text, also in Focus mode, has the display switch (Original, Translation, Side by side), a translation language list with every target language of the novel (English or Vietnamese, except the source language), and the issue count of the chapter
 AC-2. Side by side shows each source paragraph next to its translated paragraph
-AC-3. A chapter not translated in the selected language shows an empty state with a "Translate" action
-AC-4. Dictionary-check issues of the chapter are listed; selecting one highlights the source and translated paragraphs
-AC-5. A stale translation shows a notice
-AC-6. The display choice stays when moving between chapters</t>
+AC-3. A chapter not translated in the selected language shows an empty state with the actions "Translate" and "Translate manually"
+AC-4. Dictionary-check issues of the chapter are listed in a new "Translation" tab of the right panel; selecting one highlights the source and translated paragraphs
+AC-5. A stale translation shows a notice; a translation made with an older instruction shows the warning "instruction changed since this translation" and is not stale
+AC-6. The display choice stays when moving between chapters
+AC-7. One translation language per page drives the reader, the Chapters panel status (REQ-039 AC-8), and the Glossary view (REQ-037)</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4818,7 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>When the reader shows a translation (REQ-040), Edit in the page header edits that translation instead of the original, like Edit Chapter (REQ-026).</t>
+          <t>In Translation or Side by side display (REQ-040), Edit in the page header edits the translation instead of the original, like Edit Chapter (REQ-026). It also works for a chapter that is not translated or failed, so the user can translate it manually.</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
@@ -4826,11 +4833,12 @@
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>AC-1. When the reader shows a translation, Edit opens the translated title and text, one paragraph per line
+          <t>AC-1. In Translation and Side by side display, Edit opens the translated title and text, one paragraph per line, with the source paragraph read-only beside each line; for a chapter not translated or failed, each line starts empty
 AC-2. The editor has Save and Cancel; leaving with unsaved changes asks for confirmation
 AC-3. After save, the dictionary check runs again and its issues are updated
 AC-4. A saved translation is marked as edited by the user
-AC-5. Edit is refused while a pipeline is running on the novel</t>
+AC-5. Edit is refused while a pipeline is running on the novel
+AC-6. The reader empty state (REQ-040 AC-3) has a "Translate manually" action that opens the editor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(REQ027): Detect, test, and set the path of the LLM CLIs in Settings
- fix(llm): detect LLM CLIs only at app start and on Detect again [REQ-027]
- docs(llm): document LLM CLI setup [REQ-027]
- fix(llm): resolve review and test findings [REQ-027]
- feat(settings): add LLM providers section to settings [REQ-027]
- feat(llm): add LLM service, IPC and self-check [REQ-027]
- feat(llm): detect and run the LLM CLIs in main [REQ-027]
- feat(llm): add shared LLM models, settings paths and error codes [REQ-027]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -2846,13 +2846,13 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
           <t>AC-1. Settings has an LLM section listing Claude Code, Codex, and Antigravity, each shown as installed (with version) or not installed
-AC-2. Detection runs when the section opens and on demand ("Detect again")
+AC-2. Detection runs once when the app starts and again only on demand ("Detect again"); opening the section shows the last result
 AC-3. User can set the path of a CLI that is not found automatically; an invalid path is refused with a clear message
 AC-4. "Test" on an installed CLI sends a short prompt and shows OK, or the error with a suggested fix (e.g. not signed in)
 AC-5. Cloud providers (OpenAI, Anthropic, Google) are shown as "Coming soon"
@@ -5699,7 +5699,7 @@
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>Human chose Electron main in /solo-solution TH02-03 (2026-10-25). Model: app-shipped suggestions per CLI + free model id. CLIs run in an empty temp folder with tools off / read-only sandbox; text goes in the prompt.</t>
+          <t>Human chose Electron main in /solo-solution TH02-03 (2026-10-25). Model: app-shipped suggestions per CLI + free model id. CLIs run in an empty temp folder with tools off / read-only sandbox; text goes in the prompt. REQ-027 (2026-10-26, human): native executables are spawned directly (no shell), cmd.exe only for npm .cmd shims; agy gets the prompt as an argument, Claude the schema inline (replaces TH02-03 Q-02).</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(REQ028): Pick a default LLM and one per feature in Settings, with a combobox for the model
- feat(shell): show LLM CLI status in status bar and home [REQ-027]
- fix(settings): match LLM pane section spacing to General [REQ-028]
- docs(llm): document LLM per feature [REQ-028]
- fix(llm): resolve review and test findings [REQ-028]
- feat(settings): add models per feature section to LLM settings [REQ-028]
- feat(components): add combobox form component [REQ-028]
- feat(llm): add default and per-feature LLM settings and resolver [REQ-028]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -2893,7 +2893,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>Human chose Electron main in /solo-solution TH02-03 (2026-10-25). Model: app-shipped suggestions per CLI + free model id. CLIs run in an empty temp folder with tools off / read-only sandbox; text goes in the prompt. REQ-027 (2026-10-26, human): native executables are spawned directly (no shell), cmd.exe only for npm .cmd shims; agy gets the prompt as an argument, Claude the schema inline (replaces TH02-03 Q-02).</t>
+          <t>Human chose Electron main in /solo-solution TH02-03 (2026-10-25). Model: app-shipped suggestions per CLI + free model id. CLIs run in an empty temp folder with tools off / read-only sandbox; text goes in the prompt. REQ-027 (2026-10-26, human): native executables are spawned directly (no shell), cmd.exe only for npm .cmd shims; agy gets the prompt as an argument, Claude the schema inline (replaces TH02-03 Q-02). REQ-028 (2026-10-26): settings.llm.default + llm.features (missing = Use default); resolveLlm / formatLlmChoice shared, LlmService.runForFeature → LLM_NOT_AVAILABLE; TH04 run dialogs (REQ-031, REQ-038, REQ-039) use them and the deep link /settings/llm#settings-llm-feature-&lt;key&gt;, so REQ-028 AC-4 and the dialog side of AC-5 are checked in TH04 (human).</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(REQ033): Review world issues by reason and severity, then merge the world when no error is open
- docs(analysis): update review severity, world conflicts and merge rules [REQ-033]
- feat(analysis): review world issues by reason and severity; errors block merge [REQ-033]
- docs(analysis): document analysis review and merge [REQ-033]
- fix(analysis): show the raw type of an entity outside the ontology in the fix dialog [REQ-033]
- fix(analysis): resolve review and test findings [REQ-033]
- feat(analysis): review chapter issues and merge the world [REQ-033]
- feat(analysis): check conflicts and apply review edits to chapter results [REQ-033]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -4387,7 +4387,7 @@
         <is>
           <t>AC-1. While a run is active, the run pill shows the current chapter and step, chapters done / total and the failed count, with Cancel
 AC-2. Each chapter has an analysis status: not analysed, clean, has issues, reviewed, stale, or failed; the timeline shows "analysed n / N" with the stale, failed and pending-merge counts
-AC-3. Failed chapters are listed in the Review view with their error; "Retry failed" starts a run on them
+AC-3. Failed chapters are not listed in the Review view; the timeline shows them as failed, and the run dialog's missing mode analyses them again (REQ-031 AC-2)
 AC-4. A chapter edited, merged, or split after analysis shows stale or not analysed until it is analysed again; stale results stay in the world, marked stale; results of deleted chapters leave the world
 AC-5. Stale is found by the chapter file name (content hash) first, then by the chapter index
 AC-6. The library inspector shows "Analysed n / N" chapters instead of "Coming soon"; the library Analysed filter is enabled (fully, partly, or not analysed)</t>
@@ -4417,7 +4417,7 @@
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>After Candidates and Predicates, code checks the result of every chapter. Chapters without issues are clean and are not reviewed. Chapters with issues are listed in the Review queue; when every issue is resolved, the user merges and the world (world.json) is rebuilt from the results of all clean and reviewed chapters.</t>
+          <t>After Candidates and Predicates, code checks the result of every chapter, and the results of all analysed chapters together for conflicts. Each issue is an error or a warning. The Review view lists the issues of all analysed chapters, grouped by reason; when no error is open, the user merges and the world (world.json) is rebuilt from the results of all analysed chapters.</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -4427,19 +4427,19 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>AC-1. Code checks every chapter result: entity names and words exist in the chapter text, quotes exist, types and predicates are in the ontology, values are allowed, and there are no conflicts (for example one name with two types)
-AC-2. A chapter without issues is clean and is not shown for review
-AC-3. The Review queue lists the issues of the chapters with issues, grouped by chapter, each with its reason and the chapter text around the words or quote highlighted
+          <t>AC-1. Code checks every chapter result: entity names and words exist in the chapter text, quotes exist, types and predicates are in the ontology, values are present and allowed, labels are present; it checks the results of all analysed chapters together for conflicts: one name with two types, an alias that is another entity's name, and two values of a single-value predicate for one entity, also across chapters
+AC-2. Each issue has a severity. Error: words or quote not found, entity type or predicate not in the ontology, entity not found, type not allowed, value missing. Warning: value not allowed, label missing, name, alias and value conflicts
+AC-3. The Review view lists the issues of all analysed chapters, grouped by reason, errors first; an entity issue shows the type icon, name and aliases; a fact issue shows the subject, predicate, object or value, label and the fact with its chapter and the words highlighted; a conflict is one issue at world level that lists its chapters
 AC-4. Matching with the chapter text ignores only differences in case, Unicode form, whitespace, and quote/dash style
-AC-5. For each issue the user can reject the item, fix it within the ontology (it is checked again), or accept it when only the words or quote are not found; the fix is saved in that chapter's result
-AC-6. Merge is enabled only when no chapter has an open issue; it rebuilds the world from the results of all clean and reviewed chapters
-AC-7. Analysing a chapter again replaces its result and its previous review; its new issues must be resolved before the next merge
-AC-8. User can filter issues by status, type, and chapter</t>
+AC-5. For each issue the user can reject the items, fix them (entity: name, type, aliases; fact: subject, predicate, object or value, label, fact text) and they are checked again, or accept a warning; an error cannot be accepted; the edit is saved in the results of all the chapters of the issue
+AC-6. Merge is enabled only when no error is open; open warnings are merged as they are; it rebuilds the world from the results of all analysed chapters
+AC-7. Analysing a chapter again replaces its result and its previous review; its new errors must be resolved before the next merge
+AC-8. User can filter issues by severity, status, type, and chapter</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(REQ034): View world graph and edit it in an overlay kept across runs and merges
- docs(analysis): document the novel world and the world overlay [REQ-034, REQ-035]
- fix(analysis): mark only the edited fact of a chapter, plural merge result [REQ-034, REQ-035]
- fix(analysis): undo deletes without losing edits, fit the table, plural aliases [REQ-035]
- fix(analysis): resolve review and test findings [REQ-034, REQ-035]
- feat(analysis): edit the world in an overlay kept across runs and merges [REQ-035]
- feat(analysis): show occurrences, a relationship filter and the merge time in the world [REQ-034]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -4476,7 +4476,7 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -4525,7 +4525,7 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2. Approve</t>
+          <t>4. Done</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">

</xml_diff>

<commit_message>
feat(REQ038): Translate the glossary with an LLM in a background pipeline, batched by entity
- docs(translation): mark REQ-038 done [REQ-038]
- docs(translation): glossary translation pipeline [REQ-038]
- fix(translation): group glossary entities once per run [REQ-038]
- feat(translation): notify glossary run counts and show its blocked reasons [REQ-038]
- feat(translation): run the glossary translation pipeline with plan, start and cancel [REQ-038]
- feat(translation): batch glossary names by entity and ask the LLM [REQ-038]

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/_docs/0.requirements-analysis.xlsx
+++ b/_docs/0.requirements-analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sources\_datntdev.projects.dreamer-studio\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00B7890-1C4F-4468-8CBD-5EAFFB08F9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEDFC74B-972B-49D9-8CBE-706110649702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19080" yWindow="34710" windowWidth="34560" windowHeight="18690" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12330" yWindow="34710" windowWidth="34560" windowHeight="18690" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capacity Catalog" sheetId="1" r:id="rId1"/>
@@ -4815,7 +4815,7 @@
         <v>65</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>353</v>

</xml_diff>